<commit_message>
Add bilingual personal information categories
</commit_message>
<xml_diff>
--- a/spib_en_fr.xlsx
+++ b/spib_en_fr.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA51"/>
+  <dimension ref="A1:AA50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,6 +569,7 @@
           <t>PSU 901</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>psu901</t>
@@ -639,6 +640,7 @@
           <t>Information may be shared with other government institutions during consultations required to process and respond to formal requests made under the Acts. Information may be shared with the Office of the Privacy Commissioner during investigations, refer to Privacy Complaints and Investigations – OPC PPU 005 and Privacy Commissioner Ad Hoc – Complaints and Investigations – OPC PPU 008 . Information may be shared with the Office of the Information Commissioner during investigations, refer to Complaint Investigations – OIC PPU 3100 and Ad Hoc Information Commissioner Complaint Investigations – OIC PPU 123 . Personal information may be shared with a government institution providing internal support services in accordance with section 29.2 of the Financial Administration Act. For information about the internal support services used, please contact the institution’s Access to Information and Privacy Coordinator. The information may be used for planning and evaluation purposes. Depersonalized and aggregated information is used to report to Parliament on the administration of the Access to Information Act and the Privacy Act.  |  Links: Privacy Complaints and Investigations – OPC PPU 005 (https://www.priv.gc.ca/au-ans/atip-aiprp/infosource_e.asp); Privacy Commissioner Ad Hoc – Complaints and Investigations – OPC PPU 008 (https://www.priv.gc.ca/au-ans/atip-aiprp/infosource_e.asp); Complaint Investigations – OIC PPU 3100 (http://www.oic-ci.gc.ca/eng/info-source.aspx); Ad Hoc Information Commissioner Complaint Investigations – OIC PPU 123 (http://www.oic-ci.gc.ca/eng/info-source.aspx)</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -696,6 +698,7 @@
           <t>PSU 931</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>psu931</t>
@@ -766,6 +769,7 @@
           <t>Information may be shared with Public Works and Government Services Canada (Receiver General for Canada) for payment purposes refer to Receiver General Payments - PWGSC PCU 712. Where applicable, information may be shared with the Bank of Canada and financial institutions of foreign countries for transactions purposes. In some cases, the SIN and other information is shared with the Canada Revenue Agency and the Province of Quebec, and is used for data matching purposes, including income verification, refer to Individual Returns and Payment Processing – CRA PPU 005 and Business Returns and Payment Processing – CRA PPU 047 . Information may be used or disclosed for financial reporting and program evaluation.  |  Links: Individual Returns and Payment Processing – CRA PPU 005 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html); Business Returns and Payment Processing – CRA PPU 047 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html)</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -823,6 +827,7 @@
           <t>PSU 932</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>psu932</t>
@@ -893,6 +898,7 @@
           <t>Information may be shared with Public Works and Government Services Canada (Receiver General for Canada) to process payments to the government institution; refer to Receiver General Payments - PWGSC PCU 712. Information may be shared with the government institution’s own financial institution. Information may be shared with financial institutions of foreign countries for transactions purposes. Information may also be shared with collection agencies for debt recovery purposes. In some cases, the SIN and other information is shared with the Canada Revenue Agency and the Province of Quebec, and is used for data matching purposes, including income verification, refer to Individual Returns and Payment Processing – CRA PPU 005 and Business Returns and Payment Processing – CRA PPU 047 . Information may be used or disclosed for financial reporting and program evaluation.  |  Links: Individual Returns and Payment Processing – CRA PPU 005 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html); Business Returns and Payment Processing – CRA PPU 047 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html)</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -950,6 +956,7 @@
           <t>PSU 940</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>psu940</t>
@@ -980,6 +987,9 @@
           <t>Le fichier décrit l’information utilisée à l’appui d’un programme de cartes d’achats d’une institution. Les cartes d’achat sont utilisées pour acquérir et payer des biens et des services, mais ne servent pas pour les dépenses liées aux voyages ou pour les dépenses liées à l’opération et à l’entretien de véhicules. Les renseignements personnels peuvent comprendre le nom du détenteur d’une carte, les coordonnées, la langue, le numéro d’identification d’employé, le numéro de la carte, la date d’expiration, la limite de crédit, et les renseignements relatifs aux vérifications ou à la conformité aux règles, et aux enquêtes.</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>Individuals who apply for an acquisition card and those who are issued such cards.</t>
@@ -1005,6 +1015,7 @@
           <t>Information may be shared with Public Works and Government Services Canada to monitor the operation of the acquisition card program and to take corrective action when required. Information may also be shared with the private sector card issuer, namely, financial institutions. The information may be also be used or disclosed for program evaluation, enforcement (refer to Security Incidents and Privacy Breaches - PSU 939 and Discipline - PSE 911 ), and for reporting to Senior Management.  |  Links: Security Incidents and Privacy Breaches - PSU 939 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu939); Discipline - PSE 911 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -1062,6 +1073,7 @@
           <t>PSU 911</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>psu911</t>
@@ -1092,6 +1104,9 @@
           <t>Ce fichier décrit des renseignements personnels sur les personnes ayant présenté des demandes d’emploi ou fourni les curricula vitae (réclamés ou non) et une correspondance connexe. Les renseignements personnels fournis par une personne dans les formulaires de demande, les curricula vitae et la correspondance peuvent comprendre son nom, ses coordonnées, sa situation et ses antécédents professionnels, ses études, son état matrimonial, sa date de naissance, son sexe, sa connaissance des langues officielles, sa situation au regard de l’équité en emploi, ses handicaps physiques, sa citoyenneté, son code d’identification de dossier personnel, son Numéro de service client, ses relevés de notes, ses lettres de recommandation et d’autres renseignements personnels.</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>Public service employees and non-public service employees seeking employment with the institution; individuals whose names have been provided as employment references, personal references, or both; and individuals referring another individual for a position.</t>
@@ -1117,6 +1132,7 @@
           <t>Relevant information would be transferred to an employee personnel record (refer to Standard Personal Information Bank Employee Personnel Record - PSE 901 ) if the individual accepts an offer of employment. This information may also be used for planning and evaluation purposes. The information may also be transferred to another institution, if the other institution is deemed to be more appropriate for potential employment opportunities for the individual. The data collected and maintained may be used for statistical purposes, training requirements, and other development opportunities. The personal information about individuals self-identified in employment equity groups may be used for statistical purposes by the institution and may be shared with the Public Service Commission of Canada, Treasury Board of Canada Secretariat, and the Canada Public Service Agency for the same purpose.  |  Links: Employee Personnel Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901)</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -1174,6 +1190,7 @@
           <t>PSE 903</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>pse903</t>
@@ -1204,6 +1221,9 @@
           <t>Les dossiers contenant les renseignements décrits dans ce fichier peuvent comprendre des rapports sur les absences et les demandes de congé, ainsi que les certificats médicaux produits pour des congés de maladie. Sur tous ces documents, on doit inscrire le Code d’identification de dossier personnel et on doit également joindre la correspondance connexe aux présences et congés. Le dossier annuel portant sur les congés et les présences peut être joint au dossier personnel d’un employé. Certains renseignements relatifs aux congés et aux présences sont présentés sous forme de modules automatisés enregistrés dans des bases de données sur le personnel de l’organisme ou du ministère (systèmes présence/temps, congés et absences.</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>Employees of the institution.</t>
@@ -1229,6 +1249,7 @@
           <t>To record attendance  and authorize leave. To support decisions on pay and benefits, such as those  concerning leave and termination of employment, to evaluate use of leave and  rates of absenteeism and to verify policy compliance. This information may be  shared for disciplinary purposes (refer to PSE  901 Employee Personnel Record and PSE  911 Discipline ).  |  Links: PSE  901 Employee Personnel Record (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#pse901); PSE  911 Discipline (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -1256,7 +1277,7 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>NDP 941</t>
+          <t>NDP 941, NDP 924</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -1281,6 +1302,8 @@
           <t>Public Standard Bank</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>psu904</t>
@@ -1301,6 +1324,8 @@
           <t>Systèmes automatisés de gestion des documents, des dossiers et de l’information</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>This standard personal information bank was terminated since all personal information retained in the systems is accounted for in personal information banks or classes of personal information of the programs or activities for which it was collected. Description terminated: December 2013.</t>
@@ -1316,6 +1341,18 @@
           <t>2013-12-01</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
           <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu904</t>
@@ -1343,6 +1380,7 @@
           <t>PSU 903</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>psu903</t>
@@ -1373,11 +1411,15 @@
           <t>Ce fichier décrit les renseignements qui sont utilisés à l’appui des fonctions de gestion de la continuité des opérations, qui comprennent l’élaboration et l’exécution, dans les délais prévus, des plans, des mesures et des procédures afin de minimiser l’interruption des services et de la disponibilité des immobilisations en cas d’urgence ou d’interruption de service. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements biographiques, les renseignements personnels de l’employé, et les renseignements médicaux. Les renseignements personnels peuvent aussi comprendre les noms et les coordonnées des personnes désignées par les employés comme personnes avec qui communiquer en cas d’urgence.</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>Employees of the government institution; Ministers and exempt staff and other personnel of offices of Ministers or Ministers of State; emergency contacts identified by employees; private sector emergency response officials and service providers; and other federal, provincial or municipal officials who may need to be contacted in the event of an emergency or disruption of services.</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>Personal information is used to plan and respond in a timely and effective manner to an emergency or to a disruption of service, to establish a list of employees, appropriate officials and their contact information. The list may be used to contact such individuals in the event of an emergency or the execution of the Business Continuity Plan. Some institutions may also require that supervisors maintain a list of direct reports, home telephone numbers and the emergency contacts identified by the direct reports. For most government institutions, personal information is collected pursuant to the Financial Administration Act (as required under the Policy on Government Security) and the Emergency Management Act. For those institutions not subject to these Acts, consult the institution’s Access to Information and Privacy Coordinator to determine the legal authority for the collection.</t>
@@ -1393,6 +1435,7 @@
           <t>Information may be shared with other federal, provincial, and municipal institutions, police, fire and other emergency response agencies as required. Some information may be shared with/described in the Standard Personal Information Banks Employee Personnel Record - PSE 901 and Occupational Health and Safety - PSE 907 . Information may also be used or disclosed for program evaluation and reporting purposes.  |  Links: Employee Personnel Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901); Occupational Health and Safety - PSE 907 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse907)</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -1450,6 +1493,7 @@
           <t>PSU 933</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>psu933</t>
@@ -1480,11 +1524,15 @@
           <t>Ce fichier décrit les renseignements liés aux plaintes déposées en vertu de la partie III de la Loi canadienne sur les droits de la personne. Les plaintes, conformément à la partie III de la Loi canadienne sur les droits de la personne, peuvent être déposées contre une organisation réglementée par le gouvernement fédéral et se rapporter à des allégations de pratiques discriminatoires fondées sur tout motif illicite. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements biographiques, les vérifications de casier judiciaire/antécédents criminels, les renseignements sur les études, le numéro d’identification d’employé, les renseignements personnels de l’employé, des renseignements sur l’équité en emploi, la nature de la plainte, les opinions et les points de vue sur, ou concernant, des individus, d’autres numéros d’identification, les renseignements médicaux, les signes distinctifs, et la signature.</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>Individuals and representatives of individuals or groups who make a complaint, respondents, and witnesses.</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>Personal information is collected pursuant to Part III of the Canadian Human Rights Act and is used to record, enquire into and resolve complaints of discrimination.</t>
@@ -1500,6 +1548,7 @@
           <t>Information may be shared with the Department of Justice Canada to provide evidence for the hearing of a complaint by the Canadian Human Rights Tribunal, the Federal Court of Canada, the Appeal Court and/or the Supreme Court of Canada. Information may be also be used or disclosed for program evaluation.</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -1557,6 +1606,7 @@
           <t>PSE 911</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>pse911</t>
@@ -1587,11 +1637,15 @@
           <t>Ce fichier décrit les renseignements personnels reliés à la demande de normes disciplinaires dans la fonction publique fédérale et les pénalités connexes, y compris le licenciement, la suspension, la rétrogradation à un poste situé dans une échelle de traitement comportant un plafond inférieur et les sanctions pécuniaires qui peuvent être appliquées en raison de manquements à la discipline ou de mauvaise conduite dans les institutions fédérales. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements biographiques, la date de naissance, le numéro d’identification d’employé, les renseignements personnels de l’employé, les renseignements financiers, les avis juridiques, les renseignements médicaux, la nature de la mauvaise conduite et la mesure disciplinaire, les opinions et les points de vue sur, ou concernant, des individus, et la signature.</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>Employees and former employees of the institution who are/were the subject of the alleged misconduct, interviewees, medical practitioners, representatives or bargaining agents, and witnesses.</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>Personal information is used to investigate alleged misconduct in government institutions and to determine the need for, and nature of, disciplinary actions. Information is also collected to support decisions on pay and benefits, attendance and leave, transfer, demotion and termination of employment. For many institutions, personal information is collected pursuant to paragraph 12(1)(c) of the Financial Administration Act. For those institutions not subject to the Act, consult the institution’s Access to Information and Privacy Coordinator to determine the legal authority for the collection.</t>
@@ -1607,6 +1661,7 @@
           <t>Some discipline measures may also be described in Standard Personal Information Bank Employee Personnel Record - PSE 901 . Information concerning grievances is described in Standard Personal Information Bank Grievances - PSE 910 . Where applicable, information may be shared with the following entities: 1) the Treasury Board of Canada Secretariat in cases of terminations / demotions, interpretation / application of cases involving important jurisprudential issues, and other special instances; 2) professional regulatory bodies, as required; and 3) law enforcement agencies in the event of an alleged criminal offence. Information may also be used or disclosed for program evaluation.  |  Links: Employee Personnel Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901); Grievances - PSE 910 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse910)</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>(1) For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator. (2) Documentation concerning a specific employee including documentation related to disciplinary action - the time limit for disposal is that specified in applicable collective agreements or a minimum of two years following the date of disciplinary action, provided no further disciplinary action has been recorded in the meantime. (3) In cases where a disciplinary action has been rescinded, the onus is on the institution to ensure that the documentation of the action concerned is immediately destroyed.</t>
@@ -1664,6 +1719,7 @@
           <t>PSU 906</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>psu906</t>
@@ -1714,6 +1770,7 @@
           <t>Individuals who report an alleged wrongdoing in the public sector as well as individuals who are alleged to have committed wrongdoing, witnesses, representatives of individuals such as union representatives and legal counsel, investigators and any other party affected by the allegation(s).</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>Personal information is used to assess, investigate, report and resolve alleged wrongdoing in the public sector. When warranted, personal information may also be used to temporarily assign other duties to a public servant and provide notice of actions taken, or proposed to be taken, to the Public Sector Integrity Commissioner on recommendations made by the Commissioner. Personal information is collected pursuant to sections 12 to 14, 22(g), 22(h), 26 and 27 of the PSDPA.</t>
@@ -1729,6 +1786,7 @@
           <t>The information may be used or disclosed for evaluation and reporting to senior management. In limited circumstances under applicable laws, reporting purposes may include reporting to the Minister, or governing council, responsible for the government institution and publicly reporting on the wrongdoing. Depersonalized and aggregated information may be shared with the Treasury Board Secretariat (Office of the Chief Human Resources Officer) for reporting purposes. Information may be shared with internal security officials, refer to Security Incidents and Privacy Breaches- PSU 939 , or other authorities having the powers to investigate under federal, provincial and municipal statutes if the investigation reveals potential fraud or other criminal wrongdoing. Information may be shared with the government institution’s labour relations division when the chief executive officer of the government institution decides to apply disciplinary measures to public servants who perpetrated wrongdoings, refer to Discipline – PSE 911 .  |  Links: Security Incidents and Privacy Breaches- PSU 939 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu939); Discipline – PSE 911 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -1786,6 +1844,7 @@
           <t>PSU 913</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>psu913</t>
@@ -1821,6 +1880,7 @@
           <t>The head of a government institution is not required, in accordance to sub-section 9(2) Privacy Act, to account for the disclosure of the information under section 8(2)(e) in the personal information bank from which the personal information was requested. Description last updated: December 2013.</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>2013-12-01</t>
@@ -1841,11 +1901,13 @@
           <t>The personal information is used to document requests received from investigative bodies pursuant to paragraph 8(2)(e) of the Privacy Act and the responses to such requests. Personal information is collected pursuant to section 8(4) of the Privacy Act and section 7 of the Privacy Regulations.</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>The information may be used or disclosed for statistical and audit purposes. Information may be shared with government institutions who are investigative bodies listed in Schedule 2 of the Privacy Regulations. Investigative bodies that receive personal information as a result of disclosures pursuant to paragraph 8(2)(e) of the Privacy Act may subsequently share such personal information with other federal investigative bodies or law enforcement agencies, for the purpose of the administration or enforcement of a law and/or the detection, prevention, or suppression of crime.</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -1903,6 +1965,7 @@
           <t>PSU 905</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>psu905</t>
@@ -1933,6 +1996,9 @@
           <t>Les dossiers contenant les renseignements décrits dans ce fichier se rapportent à l’utilisation des réseaux électroniques des institutions fédérales. Des journaux contenant le détail sur l’utilisation des réseaux sont compilés et revus par les agents appropriés de l’institution lorsqu’il y a lieu de soupçonner la non-conformité aux politiques ou qu’un réseau électronique d’une institution fédérale est soumis à un usage détourné, au sens donné à ce terme dans les politiques en la matière de l’institution intéressée ou de la Politique d’utilisation des réseaux  électroniques, ou autres instruments de politiques et orientations pertinents du Conseil du Trésor. Ces dossiers peuvent comprendre par exemple des journaux de réseau qui  établissent des liens entre le poste de travail d’un employé et une adresse du protocole Internet, les listes de sites consultés et des renseignements sur les opérations effectuées, y compris la date, l’heure, la durée et la nature de la visite ou de l’opération. Ils peuvent aussi s’étendre à de l’information sur l’usage fait de codes d’autorisation attribués à des particuliers, y compris les cas où les codes ont pu être utilisés avec succès ou non, la date, l’heure et la fréquence d’utilisation.</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>Employees of the government institution and other individuals using institutional electronic networks, including: student employees; contract staff and agency personnel; members of the public; Ministerial staff; or Members of Parliament that send e-mail to the government institution or specific individuals within the government institution.</t>
@@ -1958,6 +2024,7 @@
           <t>The information may be used to substantiate any disciplinary action taken where violation of institutional policies or the Policy on the Use of Electronic Networks is determined, and to support compliance with other relevant Treasury Board policy instruments or policy directions. This information may be shared for disciplinary purposes (refer to PSE 901 Employee Personnel Record and PSE 911 Discipline ). If an internal investigation determines that criminal actions may have taken place, the information may be shared with appropriate police authorities. This information may be used to provide reports to management. The information may also be used for research, planning, audit and evaluation purposes.  |  Links: PSE 901 Employee Personnel Record (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#pse901); PSE 911 Discipline (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2015,6 +2082,7 @@
           <t>PSE 916</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>pse916</t>
@@ -2045,6 +2113,9 @@
           <t>Les dossiers contenant des renseignements décrits dans ce fichier sont traités de façon confidentielle en ce qui touche la participation d’un employé au Programme d’aide aux employés. Ces dossiers peuvent comprendre des avis de mise en rapport volontaire ou obligatoire (connexe au rendement au travail); des dossiers de mise en rapport avec des professionnels de la santé ou un organisme de réadaptation, et les rapports et la correspondance provenant de ces derniers; les interprétations non médicales concernant les capacités ou les limites de travail de l’employé. Tous les renseignements médicaux personnels sont conservés à titre de renseignements médicaux protégés dans un fichier administré par l’Agence des services d’hygiène du travail et du milieu. Les dossiers ayant trait aux lacunes en matière de rendement de l’employé, à l’absentéisme et aux questions disciplinaires doivent être conservés dans le fichier pertinent de renseignements personnels de l’organisme ou du ministère, et non dans les dossiers du Programme d’aide aux employés.</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>Employees of the institution.</t>
@@ -2070,6 +2141,7 @@
           <t>To support decisions regarding employee assistance measures.</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2127,6 +2199,7 @@
           <t>PSE 912</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>pse912</t>
@@ -2162,6 +2235,7 @@
           <t>Bank formerly called Performance Management Reviews. Description last updated: March 2014.</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>2014-03-01</t>
@@ -2194,7 +2268,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Les renseignements peuvent être utilisés ou divulgués pour les raisons suivantes : établissement de rapports à la haute direction, évaluation, audit, gestion des talents et planification de la relève, analyse des politiques, recherche et statistique. Dans le cas des institutions faisant partie de l’administration publique centrale, les renseignements peuvent être communiqués au Secrétariat du Conseil du Trésor du Canada; voir SCT PCE 754 Programme de gestion du rendement pour les employés . Les renseignements peuvent être communiqués à d’autres programmes et activités de l’institution; voir POE 911 – Mesures disciplinaires , POE 916 – Aide aux employés , POE 901 – Dossier personnel d’un employé , POE 910 – Griefs , POU 935 – Planification des ressources humaines , POE 907 – Santé et sécurité au travail , POE 904 – Rémunération et avantages , POE 920 – Programme de la reconnaissance , POE 902 – Dotation et POE 905 – Formation et perfectionnement .  |  Links: SCT PCE 754 Programme de gestion du rendement pour les employés (http://www.tbs-sct.gc.ca/atipo-baiprp/sfg-srg/sfg-srg02-fra.asp#SCTPCE754); POE 911 – Mesures disciplinaires (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe911); POE 916 – Aide aux employés (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe916); POE 901 – Dossier personnel d’un employé (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe901); POE 910 – Griefs (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe910); POU 935 – Planification des ressources humaines (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou935); POE 907 – Santé et sécurité au travail (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe9071); POE 904 – Rémunération et avantages (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe904); POE 920 – Programme de la reconnaissance (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe920); POE 902 – Dotation (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe9021); POE 905 – Formation et perfectionnement (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe905)</t>
+          <t>Les renseignements peuvent être utilisés ou divulgués pour les raisons suivantes : établissement de rapports à la haute direction, évaluation, audit, gestion des talents et planification de la relève, analyse des politiques, recherche et statistique. Dans le cas des institutions faisant partie de l’administration publique centrale, les renseignements peuvent être communiqués au Secrétariat du Conseil du Trésor du Canada; voir SCT PCE 754 Programme de gestion du rendement pour les employés . Les renseignements peuvent être communiqués à d’autres programmes et activités de l’institution; voir POE 911 – Mesures disciplinaires , POE 916 – Aide aux employés , POE 901 – Dossier personnel d’un employé , POE 910 – Griefs , POU 935 – Planification des ressources humaines , POE 907 – Santé et sécurité au travail , POE 904 – Rémunération et avantages , POE 920 – Programme de la reconnaissance , POE 902 – Dotation et POE 905 – Formation et perfectionnement .  |  Links: SCT PCE 754 Programme de gestion du rendement pour les employés (http://www.tbs-sct.gc.ca/atipo-baiprp/sfg-srg/sfg-srg02-fra.asp#SCTPCE754); POE 911 – Mesures disciplinaires (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe911); POE 916 – Aide aux employés (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe916); POE 901 – Dossier personnel d’un employé (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe901); POE 910 – Griefs (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe910); POU 935 – Planification des ressources humaines (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou935); POE 907 – Santé et sécurité au travail (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe907); POE 904 – Rémunération et avantages (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe904); POE 920 – Programme de la reconnaissance (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe920); POE 902 – Dotation (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe902); POE 905 – Formation et perfectionnement (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe905)</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -2289,11 +2363,15 @@
           <t>Ce dossier décrit les renseignements sur l’emploi d’une personne dans les institutions fédérales. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements biographiques (y compris le service militaire, les désignations ou certifications professionnelles), la citoyenneté, la date et le lieu de naissance, les renseignements sur les études, le numéro d’identification d’employé, des renseignements sur l’équité en emploi, les pouvoirs délégués accordés ou les biens prêtés aux employés (p. ex., les pouvoirs de dotation ou de signature de documents financiers, l’utilisation de matériel institutionnel), les réaménagements des horaires de travail (p. ex., télétravail, semaine de travail comprimée), les renseignements liés à la pension de retraite, les avantages sociaux, la formation et le perfectionnement, les griefs, les incidents de sécurité, toute autre exigence liée à l’emploi (p. ex., permis de port d’arme à feu, autorisations de sécurité, renseignements sur le passeport/visa), les renseignements financiers (pour l’administration de la paye), les renseignements médicaux (y compris tous les besoins spéciaux déterminés dans le cadre de l’obligation de prendre des mesures d’adaptation, ou en cas d’urgence), d’autres numéros d’identification, la signature et le numéro d’assurance sociale (NAS). Les informations sur l'équité en matière d'emploi ne seront utilisées qu'aux fins principales, et non pour les utilisations compatibles énumérées.</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>Current and former employees of government institutions, emergency contacts of employees, and may also include spouses, dependants, and beneficiaries.</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>Personal information is used to facilitate personnel administration in the employing institution and to ensure continuity and accuracy when an employee is transferred to another institution. For most government institutions, personal information is collected under the authority of the Public Service Employment Act (PSEA). For those institutions not subject to the (PSEA), consult the institution’s Access to Information and Privacy Coordinator to determine the legal authority for the collection. The Social Insurance Number is collected pursuant to the Income Tax Act.</t>
@@ -2309,6 +2387,7 @@
           <t>Information is disclosed to Canada Revenue Agency refer to Individual Returns and Payment Processing – CRA PPU 005 and to the Province of Quebec (where applicable) for income tax purposes. Information is also disclosed to Employment and Social Development Canada (ESDC) for employment insurance and pension purposes. Information may also be disclosed to Public Works and Government Services Canada (PWGSC) to facilitate payment of salary including direct deposit refer to Bank Public Service Compensation Systems - PWGSC PCE 705 . Where applicable, information may also be disclosed to various provincial health insurance plans or third-party group insurance companies. Information may be used to confirm the identity of employees for access to government and institutional information technology infrastructure. Where applicable, information may be disclosed to Shared Services Canada (SSC). Selected information is shared with previous employers for the purpose of finalizing payments, including retroactive payments and the recovery of outstanding amounts owing to the Crown. Information may be used for general human resource management purposes, including to verify and report on policy compliance. In instances of suspected non-compliance, information may be disclosed to the institution’s security and/or staff relations officials for further investigations or disciplinary actions (refer to PSU 939 Security Incidents and Privacy Breaches and PSE 911 Discipline ). Information may also be used or disclosed for program evaluation purposes.  |  Links: Individual Returns and Payment Processing – CRA PPU 005 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html); Public Service Compensation Systems - PWGSC PCE 705 (http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/ressources-resources/infosource-eng.html); PSU 939 Security Incidents and Privacy Breaches (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#psu939); PSE 911 Discipline (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2324,9 +2403,15 @@
           <t>98/005 and 98/018</t>
         </is>
       </c>
+      <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr">
         <is>
           <t>PRN 920</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>NDP 920</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2356,6 +2441,7 @@
           <t>PSE 918</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>pse918</t>
@@ -2386,6 +2472,9 @@
           <t>Les dossiers contenant les renseignements décrits dans ce fichier comprennent des renseignements personnels sur les employés, notamment sur leurs études; leurs antécédents professionnels et leurs projets de carrière; leur formation et leur perfectionnement. Tous ces renseignements ont été recueillis au moyen de questionnaires ou d’entrevues, ou compilés à partir de leurs dossiers ou des systèmes de données automatisés. Les répondants, qui sont libres de fournir ces renseignements, indiquent leur sexe et s’ils sont autochtones, handicapés ou font partie d’une minorité visible. Le Code d’identification de dossier personnel peut servir à identifier les employés lorsque les institutions fédérales ne peuvent pas utiliser un questionnaire anonyme ou lorsqu’il est nécessaire d’avoir ces indicatifs afin de pouvoir trouver le dossier de l’employé.</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>Employees of the institution.</t>
@@ -2403,7 +2492,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Ces dossiers ont pour but de recueillir toute la documentation nécessaire à la mise en œuvre de la politique relative à l’équité en matière d’emploi pour toutes les institutions fédérales. C’est grâce à ces renseignements qu’il est possible d’avoir toutes les données au sujet des employés, présentées selon leur sexe et leur groupe cible (femmes, autochtones et personnes handicapées et personnes faisant partie de minorités visibles). Ces renseignements sont utilisés afin de réaliser un profil personnel des employés et de comparer la situation des membres des groupes cibles avec celles des autres groupes au sein des ministères et organismes fédéraux et avec leurs homologues sur le marché du travail. Le Code d’identification de dossier personnel peut servir à établir un lien entre les renseignements contenus dans ce fichier et ceux conservés dans un autre fichier comprenant des renseignements sur les employés (p. ex., le Système d’information pour la gestion du personnel) et ce, à des fins statistiques et lorsque la conservation de tels renseignements est conforme aux usages pour lesquels les renseignements personnels ont été recueillis. Il est possible d’obtenir des données d’auto-identification des dossiers institutionnels qui sont décrits dans le Fichier de renseignements personnels Dotation – POE 902 .  |  Links: Dotation – POE 902 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe9021)</t>
+          <t>Ces dossiers ont pour but de recueillir toute la documentation nécessaire à la mise en œuvre de la politique relative à l’équité en matière d’emploi pour toutes les institutions fédérales. C’est grâce à ces renseignements qu’il est possible d’avoir toutes les données au sujet des employés, présentées selon leur sexe et leur groupe cible (femmes, autochtones et personnes handicapées et personnes faisant partie de minorités visibles). Ces renseignements sont utilisés afin de réaliser un profil personnel des employés et de comparer la situation des membres des groupes cibles avec celles des autres groupes au sein des ministères et organismes fédéraux et avec leurs homologues sur le marché du travail. Le Code d’identification de dossier personnel peut servir à établir un lien entre les renseignements contenus dans ce fichier et ceux conservés dans un autre fichier comprenant des renseignements sur les employés (p. ex., le Système d’information pour la gestion du personnel) et ce, à des fins statistiques et lorsque la conservation de tels renseignements est conforme aux usages pour lesquels les renseignements personnels ont été recueillis. Il est possible d’obtenir des données d’auto-identification des dossiers institutionnels qui sont décrits dans le Fichier de renseignements personnels Dotation – POE 902 .  |  Links: Dotation – POE 902 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe902)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2411,6 +2500,7 @@
           <t>The government institution may collect data for statistical purposes, for purposes relating to individuals, or for both. Personal data are released to the Treasury Board of Canada Secretariat for statistical purposes only (refer to Central Personal Information Bank Employment Equity Data Bank - TBS PCE 739 ). The information gathered will be used for institutional purposes in the government’s employment equity program to identify and eliminate systemic discrimination in employment and to introduce temporary special measures to ensure that target groups participate in and are equitably represented in the federal public service. It may also be used for policy and planning purposes related to employment equity.  |  Links: Employment Equity Data Bank - TBS PCE 739 (http://www.tbs-sct.gc.ca/atipo-baiprp/sfg-srg/sfg-srg02-eng.asp)</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2468,6 +2558,7 @@
           <t>PSU 902</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>psu902</t>
@@ -2475,7 +2566,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>poe902</t>
+          <t>pou902</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2498,6 +2589,9 @@
           <t>Les dossiers contenant les renseignements décrits dans ce fichier comprennent la correspondance générale du ministre ou du secrétaire d’État, de leur personnel ainsi que celle d’autres cadres supérieurs au sein de l’institution. Les dossiers utilisés pour préparer les réponses à la correspondance reçue peuvent contenir des renseignements personnels particuliers qui sont fournis parfois par des agents de l’institution afin de donner suite aux questions et aux préoccupations soulevées dans le courrier d’arrivée. Les renseignements personnels peuvent comprendre le nom du correspondant, ses coordonnées ainsi que d’autres renseignements que l’expéditeur et/ou le répondant a inclus dans la correspondance.</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>General public, Members of Parliament, and officials representing other levels of government or international governments and agencies, external organizations and/or businesses.</t>
@@ -2523,6 +2617,7 @@
           <t>Incoming correspondence may be forwarded to other federal or provincial institutions for a full or partial response if it is determined by the receiving institution that the issue(s) contained within the correspondence fall under the jurisdiction of, and should be addressed by, the other institution(s). In some cases, incoming correspondence and the response may be copied to another federal or provincial institution where the correspondence impacts on their roles and responsibilities. The information may be used in an aggregate format to report on system use, growth of the information collection, etc. The Executive Correspondence Management System may be integrated with the institution’s Automated Document, Records and Information Management System.</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2560,7 +2655,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe902</t>
+          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou902</t>
         </is>
       </c>
     </row>
@@ -2580,6 +2675,7 @@
           <t>PSU 942</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>psu942</t>
@@ -2610,11 +2706,15 @@
           <t>Ce fichier décrit des renseignements personnels inhérents à la fonction et aux activités d’évaluation d’une institution fédérale. Les renseignements personnels dont il est question peuvent comprendre le nom, les coordonnées, des données démographiques, des renseignements financiers, des numéros d’identification, le sexe, des titres de poste, ainsi que des opinions et des points de vue sur, ou concernant, des individus et recueillis, dans certains cas, avec le consentement éclairé des personnes visées.</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>Program participants, managers, employees, or partners of the program or institution, including government representatives from other jurisdictions, representatives of businesses and private sector organizations, academics or other experts in the program area, and other stakeholders including members of the general public.</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>Personal information is used in data collection and analysis when undertaking evaluations. In some cases, a limited amount of personal information, (typically names and /or titles of academics or other experts) may appear in evaluation reports where informed consent has been given by the person or persons to whom the information relates. For many institutions, information is collected pursuant to sections 7 and 42.1 of the Financial Administration Act. For those not subject to the Act, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority.</t>
@@ -2630,6 +2730,7 @@
           <t>Information may be shared with the deputy head of the institution, the government institution Evaluation Committee, and program managers. Information may be also be shared with (1) other government institutions or other partners involved in managing or delivering the program and in undertaking the evaluation; (2) Treasury Board Secretariat officials; and (3) consultants performing evaluation work on behalf of the institution. Final evaluation reports are made publicly available.</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2722,6 +2823,9 @@
           <t>Ce fichier décrit l’information sur les employés fédéraux de la catégorie EX qui s’inscrivent à l’outil de gestion des talents des cadres supérieurs. Les renseignements personnels peuvent comprendre le nom, les coordonnées de la personne et du superviseur, le numéro d’identification de l’employé, de l’information sur l’équité en emploi, des renseignements biographiques, des renseignements sur les études, des renseignements personnels de l’employé, la date de naissance, le sexe, les opinions et points de vue sur, ou concernant, des individus, la photo et la signature.</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>Employees at the EX-01 to EX-02 category and levels who choose to register for this tool. The tool is mandatory for employees at the EX-03, EX-04 and EX-05 levels (Assistant Deputy Minister levels).</t>
@@ -2747,6 +2851,7 @@
           <t>Information collected for executives who are at the ADM or equivalent level may be shared with the Clerk of the Privy Council’s Committee of Senior Officials. Information may also be shared with/described in the Standard Personal Information Banks: Employee Performance Management Program – PSE 912 , Training and Development - PSE 905 , and Human Resources Planning - PSU 935 . Information may also be used or disclosed for program evaluation.  |  Links: Employee Performance Management Program – PSE 912 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse912); Training and Development - PSE 905 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse905); Human Resources Planning - PSU 935 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu935)</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2804,6 +2909,7 @@
           <t>PSU 918</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>psu918</t>
@@ -2834,6 +2940,9 @@
           <t>Sont décrits dans ce fichier les renseignements recueillis à l’appui des nominations du gouverneur en conseil dans les institutions fédérales. Les renseignements personnels recueillis peuvent comprendre: le nom complet de la personne, ses coordonnées, sa langue officielle de préférence, sa date de naissance, son pays natal, sa citoyenneté, son sexe, sa situation de famille, son numéro d’assurance sociale (NAS), un numéro d’identification exclusif (p. ex., un numéro d’employé unique), les modalités de sa nomination, y compris sa rémunération (p. ex., traitement, honoraires, indemnité quotidienne) et ses avantages sociaux, sa signature, ses limitations physiques et toute autre information médicale pertinente, des photographies ou d’autres enregistrements visuels, sa scolarité, sa situation d’emploi, ses antécédents de travail, ses affiliations professionnelles, de l’information sur ses cartes de crédit et son établissement bancaire, sa cote de sécurité au gouvernement, des données biographiques (y compris des renseignements sur les membres de sa famille), toute déclaration de conflit d’intérêts, des lettres de référence/de recommandation, la date de nomination, la durée de la nomination et la date de démission, s’il y a lieu.</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>Current and former appointees and their family members.</t>
@@ -2859,6 +2968,7 @@
           <t>Personal information about the appointee is contained in the Order in Council document which includes full name, contact information, the position to which s/he is being appointed, the length and tenure of the appointment, and the terms and conditions of the appointment (e.g., remuneration, benefits, vacation leave, etc.). This information is provided by the Privy Council Office to the institution (refer to Governor in Council Personnel Records - PCO PPU 020 ). Governor in Council Personnel Records - PCO PPU 020). Additionally, this information may be used in the preparation of reports for senior management and broader audiences (e.g., Annual Reports) and communications materials (e.g., press releases, biographies, etc.) that may be disseminated in multiple formats, including the institution’s website. In some instances, the Privy Council Office receives notes and performance ratings to support the conduct of performance evaluations of selected individuals (refer to Governor in Council Personnel Records - PCO PPU 020 ). The Social Insurance Number (SIN) is collected pursuant to the Income Tax Act (refer to Individual Returns and Payment Processing – CRA PPU 005 ) and, where applicable, the Province of Quebec Income Tax Act.  |  Links: Governor in Council Personnel Records - PCO PPU 020 (http://www.pco-bcp.gc.ca/index.asp?lang=eng&amp;page=information&amp;sub=publications&amp;doc=info-source/index-eng.htm); Governor in Council Personnel Records - PCO PPU 020 (http://www.pco-bcp.gc.ca/index.asp?lang=eng&amp;page=information&amp;sub=publications&amp;doc=info-source/index-eng.htm); Individual Returns and Payment Processing – CRA PPU 005 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html)</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -2916,6 +3026,7 @@
           <t>PSE 910</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>pse910</t>
@@ -2956,6 +3067,7 @@
           <t>Pour les institutions assujetties à la Loi sur les relations de travail dans la fonction publique, l’article 208 de la Loi confère à un employé le droit de présenter un grief individuel à moins qu’une procédure administrative de réparation ne soit prévue dans une loi fédérale, distincte de la Loi canadienne sur les droits de la personne.</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>Current and past employees of government institutions, their representatives or bargaining agents, and any other witness or individual who may be involved in the grievance process including individuals who serve as mediators, adjudicators, or arbitrators.</t>
@@ -2981,6 +3093,7 @@
           <t>Information concerning grievances filed under the Public Service Labour Relations Act may be shared with the Public Service Labour Relations Board (refer to Central Personal Information Banks: Applications for Extension of Time - PSLRB PCE 710 , Applications for an extension of time in respect of a grievance - PSLRB PCE 715 , Complaint/Grievance Mediation - PSLRB PCE 726 , Complaints under Section 190 of the Public Service Labour Relations Act (PSLRA) - RLT PCE 730 , and Requests for Review of Decisions – PSLRB PCE 793 . Certain complaints may be referred to mediation, adjudication, or arbitration by the Public Service Labour Relations Board (refer to Central Personal Information Banks: References of Grievances to Adjudication - PSLRB PCE 791 and Reference to Adjudication of Individual Grievances - PSLRB PCE 792 ). In these cases, information may be disclosed to individuals who are appointed by the Public Service Labour Relations Board or by a government institution to serve as mediators, adjudicators or arbitrators. Full-text versions of decisions are posted on the Public Service Labour Relations Board website. In some cases, information may be shared with the Canadian Human Rights Commission where a party to a grievance raises an issue involving the interpretation or application of the Canadian Human Rights Act within the context of a request for arbitration of the grievance. Aggregate information may be used or disclosed for annual reporting purposes. Some information about grievances may also be shared with/described in Standard Personal Information Banks Employee Personnel Record - PSE 901 and Discipline - PSE 911 . Information may also be used or disclosed for evaluation purposes.  |  Links: Applications for Extension of Time - PSLRB PCE 710 (http://www.pslrb-crtfp.gc.ca/reports/infosource_e.asp); Applications for an extension of time in respect of a grievance - PSLRB PCE 715 (http://www.pslrb-crtfp.gc.ca/reports/infosource_e.asp); Complaint/Grievance Mediation - PSLRB PCE 726 (http://www.pslrb-crtfp.gc.ca/reports/infosource_e.asp); Complaints under Section 190 of the Public Service Labour Relations Act (PSLRA) - RLT PCE 730 (http://www.pslrb-crtfp.gc.ca/reports/infosource_e.asp); Requests for Review of Decisions – PSLRB PCE 793 (http://www.pslrb-crtfp.gc.ca/reports/infosource_e.asp); References of Grievances to Adjudication - PSLRB PCE 791 (http://www.pslrb-crtfp.gc.ca/reports/infosource_e.asp); Reference to Adjudication of Individual Grievances - PSLRB PCE 792 (http://pslrb-crtfp.gc.ca/reports/intro_e.asp); Employee Personnel Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901); Discipline - PSE 911 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -3038,6 +3151,7 @@
           <t>PSE 919</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>pse919</t>
@@ -3088,6 +3202,7 @@
           <t>Employees and other persons working for a government institution, or other persons involved in alleged occurrences of harassment and violence in federal institutions.</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>Information is used to prevent, resolve and investigate harassment and violence notices of occurrence (including through early resolution and conciliation processes), ensuring that all parties involved are treated with respect and dignity throughout the process. Procedural fairness is upheld by providing the principal party and responding party with the opportunity to be heard, ensuring that decisions are made impartially and maintaining transparency in the resolution process.</t>
@@ -3165,6 +3280,7 @@
           <t>PSU 908</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>psu908</t>
@@ -3195,11 +3311,15 @@
           <t>Ce fichier décrit les renseignements liés à la fourniture de breuvages, de repas, de visites guidées ou d’autres divertissements remboursés par les institutions fédérales. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements personnels de l’employé, le numéro d’identification d’employé et les renseignements financiers.</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>Employees of the government institution who incur hospitality expenses, their spouses, other attendees, private sector hospitality providers and/or other individuals who may be paid out of the Consolidated Revenue Fund (i.e. who receive a fee, honorarium or per diem allowance).</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>Personal information is used to administer the hospitality expenses and reimbursements of government institutions. For most government institutions, personal information is collected pursuant to the Financial Administration Act. For those institutions not subject to the Act, consult the institution’s Access to Information and Privacy Coordinator to determine the legal authority for the collection.</t>
@@ -3215,6 +3335,7 @@
           <t>Where applicable, hospitality expenses incurred by the Minister, Parliamentary Secretary, exempt staff, and by senior level employees (i.e. Deputy Minister, Associate Deputy Minister, Assistant Deputy Minister, and equivalent) may be proactively disclosed on government institutions’ websites. Information may be shared with/described in Standard Personal Information Bank Accounts Payable - PSU 931 . Information may also be used or disclosed for program evaluation and reporting purposes.  |  Links: Accounts Payable - PSU 931 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu931)</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -3240,6 +3361,7 @@
           <t>PRN 933, PRN 935</t>
         </is>
       </c>
+      <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr">
         <is>
           <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu908</t>
@@ -3302,6 +3424,9 @@
           <t>Ce fichier décrit l’information liée à la gestion salariale et à la planification des ressources humaines, ce qui comprend les fonctions de compte rendu et d’établissement des prévisions. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements biographiques, les renseignements sur l’éducation, le numéro d’identification de l’employé, les renseignements sur l’équité en emploi, les renseignements personnels de l’employé, et les opinions et points de vue sur, ou concernant, des individus.</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>Current and former employees of government institutions, job applicants, students, casual and contract employees, and Interchange Canada participants.</t>
@@ -3327,6 +3452,7 @@
           <t>Personal information may be shared with other government institutions in cases of transfer of section of the public service under the Public Service Rearrangement and Transfer of Duties Act. Personal information may be shared with provincial or municipal governments, and institutions thereof, or private sector institutions in cases of devolution or privatization of a program or activity. Some employee information may also be shared with/described in the Standard Personal Information Banks Employment Equity Program - PSE 918 , Employee Personal Record - PSE 901 , Pay and Benefits - PSE 904 , Staffing - PSE 902 , Training and Development - PSE 905 , and Official Languages - PSE 906 . Information may be also be used or disclosed for program evaluation.  |  Links: Employment Equity Program - PSE 918 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse918); Employee Personal Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901); Pay and Benefits - PSE 904 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse904); Staffing - PSE 902 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse902); Training and Development - PSE 905 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse905); Official Languages - PSE 906 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse906)</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator</t>
@@ -3384,6 +3510,7 @@
           <t>PSU 941</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>psu941</t>
@@ -3424,6 +3551,7 @@
           <t>Les renseignements personnels qui se trouvent dans les documents de l’institution peuvent être divulgués au Bureau du vérificateur général pour des études ou des vérifications.</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>Employees and former employees of the institution, contractors, representatives of companies.</t>
@@ -3449,6 +3577,7 @@
           <t>Information may be shared with responsible managers, and in some cases, the government institution Audit Committee, the Audit Committee of the Board of Directors, the Board of Directors, and/or the Office of the Auditor General. Information may be also be shared with: 1) Human Resources for disciplinary measures (refer to Discipline – PSE 911 ); 2) Security (refer to Security Incidents and Privacy Breaches – PSU 939 ); 3) Investigative personnel and law enforcement agencies in the event of an alleged criminal offence; and 4) consultants performing internal audit work on behalf of the institution’s Chief Audit Executive.  |  Links: Discipline – PSE 911 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse911); Security Incidents and Privacy Breaches – PSU 939 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu939)</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -3469,6 +3598,7 @@
           <t>99/004</t>
         </is>
       </c>
+      <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr">
         <is>
           <t>NDP 916</t>
@@ -3501,6 +3631,7 @@
           <t>PSU 915</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>psu915</t>
@@ -3541,11 +3672,13 @@
           <t>Ces renseignements peuvent être stockés sous forme papier ou électronique (p. ex., dans des bases de données ou dans des sites Web, y compris les applications de médias sociaux, etc.). Bien qu’une institution ne demande pas les adresses du protocole Internet expressément, celles-ci peuvent être saisies de manière électronique à la réception d’un courriel.</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>Employees and other individuals with access to institutional networks including individuals who have prepared information for dissemination, such as publication on the institution’s intranet, or who act as contact points within the institution.</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>Personal information is used to manage internal communications. For many institutions, personal information is collected under the authority of the Financial Administration Act, and in accordance with the Communications Policy of the Government of Canada. For those institutions not subject to the Act or the Policy, consult the institution’s Access to Information and Privacy Coordinator to determine the legal authority for the collection.</t>
@@ -3561,6 +3694,7 @@
           <t>The names, photographs, recordings and other personal information about individuals who work for the institution may be included in documentation posted on the institution’s intranet: e.g., within speeches, newsletters, etc. Information may be used or disclosed to provide statistical reports to management as well as for program evaluation.</t>
         </is>
       </c>
+      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -3618,6 +3752,7 @@
           <t>PSU 936</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>psu936</t>
@@ -3648,11 +3783,15 @@
           <t>Ce fichier décrit l’information sur les personnes qui utilisent les installations, les collections et les services de bibliothèques des institutions fédérales. Les services peuvent comprendre les prêts, les références et la recherche, ainsi que les services d’avertissement et de mises au courant, dont l’évaluation des demandes des clients quant aux nouvelles acquisitions. Les renseignements personnels peuvent comprendre le nom, les coordonnées, l’affiliation de l’organisme, le sujet de recherche, d’autres numéros d’identification, y compris le numéro de carte de l’utilisateur et sa date d’expiration, ainsi que le numéro de code à barres du client.</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>Full-and part-time, casual, and term employees of government institutions, agency employees, members of the general public, researchers, and employees of non-government institution libraries.</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>Personal information is used to support the delivery of library services of government institutions, such as identifying user preferences, researching topics, analyzing trends in information needs, processing inter-library loans, and controlling the circulation of material.</t>
@@ -3668,6 +3807,7 @@
           <t>Information may be used or disclosed for program evaluation.</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -3760,6 +3900,9 @@
           <t>Ce fichier décrit l’information recueillie par les titulaires d’une charge publique désignée (p. ex., les administrateurs généraux actuels et les anciens administrateurs généraux, les sous-ministres adjoints, les cadres supérieurs des Forces canadiennes, etc.) au sujet de la vérification des activités des lobbyistes sur demande du commissaire au lobbying. Les renseignements personnels peuvent comprendre le nom, les coordonnées, de l’information financière, des renseignements biographiques, la date et de l’heure de l’activité de communication/lobbying, ainsi que les opinions et les points de vue des individus sur le sujet.</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>Designated public office holders and lobbyists as defined in the Lobbying Act.</t>
@@ -3785,6 +3928,7 @@
           <t>Information may be made accessible to the public via the website of the Office of the Commissioner of Lobbying of Canada (refer to Information-Specific Personal Information Bank Lobbyist Registry - OCL PPU 039 ). Information may be also be used or disclosed for program evaluation.  |  Links: Lobbyist Registry - OCL PPU 039 (https://lobbycanada.gc.ca/eic/site/012.nsf/eng/00843.html)</t>
         </is>
       </c>
+      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -3842,6 +3986,7 @@
           <t>PSU 919</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>psu919</t>
@@ -3872,6 +4017,9 @@
           <t>Ce fichier décrit les renseignements personnels utilisés dans le processus d’identification et de sélection des personnes qui seront nommées aux conseils d’administration, comités et conseils de diverses institutions. Les renseignements personnels peuvent comprendre : le nom complet de la personne, ses coordonnées, sa langue officielle de préférence, sa date de naissance, son pays natal, sa citoyenneté, son sexe, sa situation de famille, son appartenance à un groupe minoritaire, son numéro d’assurance sociale (NAS), un numéro d’identification exclusif (p. ex., un numéro d’employé unique), les modalités de sa nomination, y compris sa rémunération (p. ex., traitement, honoraires, indemnité quotidienne) et ses avantages sociaux, sa signature, ses limitations physiques et toute autre information médicale pertinente, des photographies ou d’autres enregistrements visuels, sa scolarité, sa situation d’emploi, ses antécédents de travail, ses activités bénévoles, ses affiliations professionnelles, de l’information sur ses cartes de crédit et son établissement bancaire, sa cote de sécurité au gouvernement, des données biographiques (y compris des renseignements sur les membres de sa famille), toute déclaration de conflit d’intérêts, des lettres de référence/de recommandation, la date de nomination, la durée de la nomination et la date de démission, s’il y a lieu.</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>Candidates, as well as current and former members of Boards, Committees, and Councils, their family members, and individuals whose names have been provided as personal references.</t>
@@ -3897,6 +4045,7 @@
           <t>This information may be used in the preparation of reports for senior management and broader audiences (e.g., Annual Reports), planning and evaluation purposes, and communications materials (e.g., press releases, biographies, etc.) that may be disseminated in multiple formats, including the institution’s website. With consent of the individual, this information may be shared with other Government of Canada institutions for uses consistent with the mandate of the Board, Committee or Council on which personal information is collected to fill positions (Refer to Members of Boards, Committees and Councils – PSU 919 of the specific government institution). Information may be disclosed to the Canada Revenue Agency (refer to Individual Returns and Payment Processing – CRA PPU 005 ) and, where applicable, the Province of Quebec for income tax purposes. Assistance of third party service providers may be used during the selection process.  |  Links: Individual Returns and Payment Processing – CRA PPU 005 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html)</t>
         </is>
       </c>
+      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -3954,6 +4103,7 @@
           <t>PSE 907</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>pse907</t>
@@ -3961,7 +4111,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>poe9071</t>
+          <t>poe907</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3984,11 +4134,15 @@
           <t>Ce fichier décrit l’information qui est utilisée dans le but d’appuyer une activité liée à la santé et à la sécurité du travail dans une institution fédérale, y compris la prévention des accidents et des blessures ou des maladies de nature professionnelle; une autorisation de congé payé liée à un accident du travail ou une maladie professionnelle; les services d’aide aux employés; les évaluations sur l’aptitude à retourner au travail; l’obligation de prendre des mesures d’adaptation; les évaluations de santé et de nature ergonomique; les plaintes relatives à la santé et à la sécurité; l’indemnisation des accidentés; la réadaptation et le recyclage. Les renseignements personnels peuvent comprendre le nom, les coordonnées, le numéro d’identification d’employé, les renseignements personnels de l’employé, les renseignements financiers, la nature de la plainte, les renseignements médicaux, les opinions et les points de vue sur, ou concernant, des individus, et la signature.</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>Current and former employees of government institutions, including casual and contract employees; private sector health practitioners; health and safety professionals; attendants for persons requiring assistance; family members who are part of the same household and eligible for corporate rates for Wellness programs; and individuals designated as emergency contacts of employees</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>Personal information is used to administer occupational safety and health activities in government institutions, which includes the promotion of a safe and healthy workplace for employees and others, provision of corporate Wellness programs, the prevention of accidents, occupational injuries and illnesses and, where applicable, the investigation of occurrences of such injuries and illnesses. Information may be collected pursuant to paragraph 7(1)(e) and subsection 11.1 of the Financial Administration Act; sections 114 and 240 of the Public Service Labour Relations Act; Part II of the Canada Labour Code and Part XVI of the Canada Occupational Health and Safety Regulations, the Government Employees Compensation Act, and the National Joint Council Directives.</t>
@@ -4004,6 +4158,7 @@
           <t>Information may be used or disclosed for the following reasons: to support decisions related to worker’s compensation and injury-on-duty leave; as a means of preventing injuries and illnesses and subsequent disabilities arising out of, or aggravated by, conditions of work; to establish that individuals subject to certain identified occupational risks are able to continue working without detriment to their health or safety or to that of others; and to establish the conditions under which certain individuals with identified illnesses or disabilities are able to continue to work under controlled conditions. Information may be shared with private sector health care providers. Information may be used to communicate with contacts of employees in emergency situations. Information concerning occupational health evaluations including related personal medical information is retained by Health Canada in the Corporate Services Branch under medical confidential status (refer to Central Personal Information Bank: Public Service Occupational Health Program - HC PCE 701 ). Information with respect to safety and health complaints and causes of accidents/injuries for accident prevention and health protection purposes is used to support the effective administration of each institution’s safety and health activity; such information is also disclosed to the institution’s work place health and safety committee. Information is also used to process payments and charge-backs with respect to injury compensation claims. Information related to injury compensation claims, including related correspondence and amounts paid, is retained by Employment and Social Development Canada and is shared with the institution of the affected employee and, where applicable, the relevant provincial or territorial workers’ compensation board. Employment and Social Development Canada holds information pertaining to employee compensation amounts, which are charged to institutions and distributed on a cost-recovery basis (refer to Personal Information Bank: Federal Workers Compensation - ESDC PPU 032 ). Information may also be shared with Employment and Social Development Canada, specifically, with safety officers for the purposes of accident and refusal to work investigations and the stipulation of corrective measures. Information may be shared with/described in other Standard Personal Information Banks pertaining to human resources activities including: Employee Personnel Record - PSE 901 ; Attendance and Leave - PSE 903 ; Employee Assistance - PSE 916 ; Pay and Benefits - PSE 904 ; and Grievances - PSE 910 . The investigation and settlement of vehicle accidents is also described in Standard Personal Information Bank Vehicle, Ship, Boat and Aircraft Accidents - PSE 908 . Information may also be used or disclosed for planning and program evaluation purposes.  |  Links: Public Service Occupational Health Program - HC PCE 701 (https://www.canada.ca/en/health-canada/corporate/about-health-canada/activities-responsibilities/access-information-privacy/info-source-federal-government-employee-information.html#a3.14); Federal Workers Compensation - ESDC PPU 032 (http://www.esdc.gc.ca/eng/transparency/ati/reports/infosource/index.shtml); Employee Personnel Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901); Attendance and Leave - PSE 903 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse903); Employee Assistance - PSE 916 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse916); Pay and Benefits - PSE 904 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse904); Grievances - PSE 910 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse910); Vehicle, Ship, Boat and Aircraft Accidents - PSE 908 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse908)</t>
         </is>
       </c>
+      <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4041,7 +4196,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe9071</t>
+          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe907</t>
         </is>
       </c>
     </row>
@@ -4061,6 +4216,7 @@
           <t>PSE 906</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>pse906</t>
@@ -4131,6 +4287,7 @@
           <t>To support and document decisions concerning individual employees on staffing, entitlement to bilingual bonus where applicable, transfers and promotions; and to aid in determining the linguistic status of employees and auditing of the administration of official language programs. Information may be disclosed to federal government institutions, the Public Service Commission and Treasury Board of Canada Secretariat where applicable for recruitment and staffing purposes (refer to Institution-Specific Personal Information Banks: for the Public Service Commission of Canada: Executive Resourcing - PSC PCE 746 ; for Treasury Board of Canada Secretariat: Employment Equity Data Bank - TBS PCE 739 ).  |  Links: Executive Resourcing - PSC PCE 746 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Employment Equity Data Bank - TBS PCE 739 (http://www.tbs-sct.gc.ca/atipo-baiprp/sfg-srg/sfg-srg02-eng.asp)</t>
         </is>
       </c>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4188,6 +4345,7 @@
           <t>PSU 938</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>psu938</t>
@@ -4238,6 +4396,7 @@
           <t>Current and former employees of government institutions, representatives of other levels of government, representatives of the academic and business communities, members of the general public (including parents and guardians where minors are concerned), and event speakers and facilitators.</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>The information is used to enable individuals to participate in national and/or international outreach activities sponsored by government institutions. Such activities facilitate information exchanges in areas of common interest to institutions and their stakeholders and allow for the sharing of knowledge, expertise, and best practices. Personal information is collected pursuant to various federal laws and regulations. For the specific collection authority(ies), consult the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4253,6 +4412,7 @@
           <t>With notification, the proceedings of some outreach activities that are recorded may be made publicly available, including on the Internet. With consent, the information may be used to establish mailing lists to inform participants of future events or to contact individuals to seek views on issues of mutual interest. Information may be used to moderate public discussion on the social media platforms used by the institution. Information may be also be used or disclosed for program evaluation.</t>
         </is>
       </c>
+      <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4310,6 +4470,7 @@
           <t>PSE 914</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>pse914</t>
@@ -4340,11 +4501,15 @@
           <t>Ce fichier décrit les renseignements personnels liés aux demandes de permis de stationnement et aux détenteurs de permis de stationnement pour des propriétés louées par ou appartenant à des institutions fédérales. Les renseignements personnels peuvent comprendre le nom, les coordonnées à la maison et au travail, les renseignements biographiques, le numéro d’identification d’employé, les renseignements personnels de l’employé, les renseignements financiers, les renseignements médicaux (pour ceux qui demandent un stationnement pour les personnes handicapées), les renseignements d’identification du véhicule, les critères de tarification, et la signature.</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>Employees of the institution, passengers, contractors or other individuals, property owners or representatives.</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>Personal information is used for the administration of parking privileges and to authorize payroll deductions. For most government institutions, personal information is collected under the authority of the Financial Administration Act. For those institutions not subject to the Act, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority.</t>
@@ -4360,6 +4525,7 @@
           <t>Where government or other property is damaged, the accident may be reported to the Royal Canadian Mounted Police (refer to Central Personal Information Bank Protection of Personnel and Government Property - RCMP PPU 055) or to other policing authorities, or to the person(s) in charge or in control of the property. Information may be shared with Public Works and Government Services for the purpose of payroll deduction (refer to Central Personal Information Bank Public Service Compensation Systems - PWGSC PCE 705 ). Payroll deduction information may be shared with/described in Standard Personal Information Bank Pay and Benefits - PSE 904 . Information may also be used or disclosed for evaluation or reporting purposes.  |  Links: Public Service Compensation Systems - PWGSC PCE 705 (http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/ressources-resources/infosource-eng.html); Pay and Benefits - PSE 904 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse904)</t>
         </is>
       </c>
+      <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4417,6 +4583,7 @@
           <t>PSE 904</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>pse904</t>
@@ -4447,11 +4614,15 @@
           <t>Ce fichier décrit les renseignements liés à l’administration de la rémunération et des avantages sociaux au sein des institutions fédérales. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements biographiques, la date de naissance, la date du décès, le numéro d’identification d’employé, les renseignements personnels de l’employé, les renseignements financiers, et le numéro d’assurance sociale (NAS).</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>Current and former employees of government institutions.</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>Personal information is shared with Public Works and Government Services and is used to disburse salaries and allowances and to process deductions and orders for garnishment and diversion of funds. Personal information is collected under various Acts including the Financial Administration Act, the Government Employees Compensation Act, and the Public Service Labour Relations Act. The Social Insurance Number (SIN) is collected pursuant to the Income Tax Act, Canada Pension Plan, and the Employment Insurance Act, and for some institutions, the SIN is shared with Public Works and Government Services to create the Personal Record Identifier.</t>
@@ -4467,6 +4638,7 @@
           <t>Information is shared with Public Works and Government Services Canada (refer to Public Service Compensation Systems -PWGSC PCE 705 and Public Service Pensions Data Bank - PWGSC PCE 702 ). Information, including the SIN, is disclosed to the Canada Revenue Agency (refer to Individual Returns and Payment Processing – CRA PPU 005 ) and the Province of Quebec (if applicable) for taxation and pension purposes. Information may also be shared with the Department of Justice Canada to administer the Family Orders and Agreements Enforcement Assistance Act and the Garnishment, Attachment and Pension Diversion Act (refer to Family Orders and Agreements Enforcement Assistance - JUS PPU 125 and Garnishment Registry - JUS PPU 150 ). Information may be shared with third party service providers, for select institutions. Some information on pay and benefits may also be shared with/described in the Standard Personal Information Banks Employee Personnel File - PSE 901 , Grievances - PSE 910 , and Discipline - PSE 911 . Information may also be used or disclosed for program evaluation.  |  Links: Public Service Compensation Systems -PWGSC PCE 705 (http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/ressources-resources/infosource-eng.html); Public Service Pensions Data Bank - PWGSC PCE 702 (http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/ressources-resources/infosource-eng.html); Individual Returns and Payment Processing – CRA PPU 005 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html); Family Orders and Agreements Enforcement Assistance - JUS PPU 125 (http://www.justice.gc.ca/eng/trans/atip-aiprp/infosource/index.html); Garnishment Registry - JUS PPU 150 (http://www.justice.gc.ca/eng/trans/atip-aiprp/infosource/p3.html); Employee Personnel File - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901); Grievances - PSE 910 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse910); Discipline - PSE 911 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4564,6 +4736,8 @@
           <t>(1) Information may be stored in either hard copy format or electronically (e.g. in databases). (2) Some institutions have developed institution-specific security screening personal information banks. Individuals seeking access to their information in PSU 917 may also want to request that other institutional PIBs related to security screening be included in the access to information request if they have worked in or for the following departments which maintain separate PIBs: Public Services and Procurement Canada (Industry Personnel Clearance and Reliability Records – PWGSC PPU 015) ; National Defence / Canadian Armed Forces (Personnel Security Investigation File – DND PPU 834) ; Privy Council Office (Security Clearance and Assessments Bank – PCO PPE 801) ; Royal Canadian Mounted Police (Security Reliability Screening Records – RCMP PPU 065) ; and Canadian Security Intelligence Service (Employee Security – SIS PPE 815) .  |  Links: Public Services and Procurement Canada (Industry Personnel Clearance and Reliability Records – PWGSC PPU 015) (https://www.tpsgc-pwgsc.gc.ca/aiprp-atip/infosource2014-eng.html); National Defence / Canadian Armed Forces (Personnel Security Investigation File – DND PPU 834) (https://www.forces.gc.ca/en/transparency-access-info-privacy/info-source-toc.page); Privy Council Office (Security Clearance and Assessments Bank – PCO PPE 801) (http://www.pco-bcp.gc.ca/index.asp?lang=eng&amp;page=information&amp;sub=publications&amp;doc=info-source/index-eng.htm); Royal Canadian Mounted Police (Security Reliability Screening Records – RCMP PPU 065) (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/pib-frp-eng.htm); Canadian Security Intelligence Service (Employee Security – SIS PPE 815) (https://www.csis.gc.ca/tp/nfsrc-en.php)</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>Job applicants, all current and former employees (students, agency and casual employees, persons on loan, assignment or secondment, exempt staff of ministers, ministers of state and parliamentary secretaries, locally engaged staff), volunteers, contractors, foreign and domestic visitors, immediate relatives, current and former spouse/common law partner, associates, cohabitants, individuals who give character references (including neighbours), current/former employers, parents or guardians of job applicants and employees under the age of 18.</t>
@@ -4586,12 +4760,12 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Where required, personal information may be shared in accordance with the institution's enabling legislation and within the parameters of the Privacy Act, with the Royal Canadian Mounted Police ( Canadian Criminal Real Time Identification Services – RCMP OPS 1214 and Personnel Security Records – RCMP ADM 445 ) and the Canadian Security Intelligence Service ( Security Assessments/Advice Records – CSIS PPU 005 ) to conduct security screening verifications, inquiries and/or assessments in accordance with the Policy on Government Security. Information may be shared with the Canadian Human Rights Commission ( Human Rights Litigation Records – CHRC DRP 020 , Human Rights Complaints Dispute Resolution Records – CHRC DRP 010 ), the Public Service Labour Relations and Employment Board ( Complaint/Grievance Mediation Records – PSLRB ROP 579 ), Justice Canada ( Litigation Services Records – JUS 3.0.5 ) or the Security Intelligence Review Committee ( Complaints Records – SIR COM 001 ) when an individual challenges a decision to deny, suspend or revoke a the required security status or security clearance. Information may be disclosed to the Privy Council Office ( Security and Intelligence Information Files – Personal Information Bank– PCO PPU 005 ) should the individual pose a potential risk to national security or is part of a national security-related investigation. The security screening status of an individual may be shared internally within institutions with human resource officials to update the individual's personnel file ( Employee Personnel Record – PSE 901 , Governor in Council Appointments – PSU 918 , Members of Boards Committees and Councils – PSU 919 ). Information may be shared within or between government institutions for staffing purposes ( Staffing – PSE 902 ). Information may be shared within institutions with departmental security officials for issuance of access cards and badges ( Physical Access Controls PSU 907 ). Information may be shared within institutions with departmental security officials in cases of adverse information for investigation ( Security – PRN 931 or Security Incidents and Privacy Breaches – PSU 939 ). Biographical information, including name, date of birth, employment and/or educational history, may be shared with individuals or entities outside the government institution to confirm identity and conduct required inquiries or verifications including: authorized credit reporting agencies, personal and/or professional referees, and educational institutions and/or professional organizations. Information, including the results of security screening checks, may be disclosed to an individual’s manager, labour relations advisors, and/or an institutional security screening advisory board, on a need to know basis, when a decision to deny, revoke or suspend pending an investigation is being considered. Information, including completed security screening forms, the results of security screening checks and decisions made by a department may be shared between institutional security officials to enable transferability of security screening and to help ensure that individuals are not engaged by another government institution without regard to the circumstances leading to any previous denial or revocation which may have taken place in another institution. Select anonymized information may be used or disclosed for program evaluation.  |  Links: Canadian Criminal Real Time Identification Services – RCMP OPS 1214 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-eng.htm); Personnel Security Records – RCMP ADM 445 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-eng.htm); Security Assessments/Advice Records – CSIS PPU 005 (https://www.csis.gc.ca/tp/nfsrc-en.php); Human Rights Litigation Records – CHRC DRP 020 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-eng.pdf); Human Rights Complaints Dispute Resolution Records – CHRC DRP 010 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-eng.pdf); Complaint/Grievance Mediation Records – PSLRB ROP 579 (http://pslrb-crtfp.gc.ca/reports/1314/infosource_e.asp); Litigation Services Records – JUS 3.0.5 (http://www.justice.gc.ca/eng/trans/atip-aiprp/infosource/p3.html); Complaints Records – SIR COM 001 (http://www.sirc-csars.gc.ca/prddpr/is/2013/index-eng.html); Security and Intelligence Information Files – Personal Information Bank– PCO PPU 005 (http://www.pco-bcp.gc.ca/index.asp?lang=eng&amp;page=information&amp;sub=publications&amp;doc=info-source/index-eng.htm); Employee Personnel Record – PSE 901 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Governor in Council Appointments – PSU 918 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Members of Boards Committees and Councils – PSU 919 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Staffing – PSE 902 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Physical Access Controls PSU 907 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu907); Security – PRN 931 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-classes-records.html); Security Incidents and Privacy Breaches – PSU 939 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp)</t>
+          <t>Where required, personal information may be shared in accordance with the institution's enabling legislation and within the parameters of the Privacy Act, with the Royal Canadian Mounted Police ( Canadian Criminal Real Time Identification Services – RCMP OPS 1214 and Personnel Security Records – RCMP ADM 445 ) and the Canadian Security Intelligence Service ( Security Assessments/Advice Records – CSIS PPU 005 ) to conduct security screening verifications, inquiries and/or assessments in accordance with the Policy on Government Security. Information may be shared with the Canadian Human Rights Commission ( Human Rights Litigation Records – CHRC DRP 020 , Human Rights Complaints Dispute Resolution Records – CHRC DRP 010 ), the Public Service Labour Relations and Employment Board ( Complaint/Grievance Mediation Records – PSLRB ROP 579 ), Justice Canada ( Litigation Services Records – JUS 3.0.5 ) or the Security Intelligence Review Committee ( Complaints Records – SIR COM 001 ) when an individual challenges a decision to deny, suspend or revoke a the required security status or security clearance. Information may be disclosed to the Privy Council Office ( Security and Intelligence Information Files – Personal Information Bank– PCO PPU 005 ) should the individual pose a potential risk to national security or is part of a national security-related investigation. The security screening status of an individual may be shared internally within institutions with human resource officials to update the individual's personnel file ( Employee Personnel Record – PSE 901 , Governor in Council Appointments – PSU 918 , Members of Boards Committees and Councils – PSU 919 ). Information may be shared within or between government institutions for staffing purposes ( Staffing – PSE 902 ). Information may be shared within institutions with departmental security officials for issuance of access cards and badges ( Physical Access Controls PSU 907 ). Information may be shared within institutions with departmental security officials in cases of adverse information for investigation ( Security – PRN 931 or Security Incidents and Privacy Breaches – PSU 939 ). Biographical information, including name, date of birth, employment and/or educational history, may be shared with individuals or entities outside the government institution to confirm identity and conduct required inquiries or verifications including: authorized credit reporting agencies, personal and/or professional referees, and educational institutions and/or professional organizations. Information, including the results of security screening checks, may be disclosed to an individual’s manager, labour relations advisors, and/or an institutional security screening advisory board, on a need to know basis, when a decision to deny, revoke or suspend pending an investigation is being considered. Information, including completed security screening forms, the results of security screening checks and decisions made by a department may be shared between institutional security officials to enable transferability of security screening and to help ensure that individuals are not engaged by another government institution without regard to the circumstances leading to any previous denial or revocation which may have taken place in another institution. Select anonymized information may be used or disclosed for program evaluation.  |  Links: Canadian Criminal Real Time Identification Services – RCMP OPS 1214 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-eng.htm); Personnel Security Records – RCMP ADM 445 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-eng.htm); Security Assessments/Advice Records – CSIS PPU 005 (https://www.csis.gc.ca/tp/nfsrc-en.php); Human Rights Litigation Records – CHRC DRP 020 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-eng.pdf); Human Rights Complaints Dispute Resolution Records – CHRC DRP 010 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-eng.pdf); Complaint/Grievance Mediation Records – PSLRB ROP 579 (http://pslrb-crtfp.gc.ca/reports/1314/infosource_e.asp); Litigation Services Records – JUS 3.0.5 (http://www.justice.gc.ca/eng/trans/atip-aiprp/infosource/p3.html); Complaints Records – SIR COM 001 (http://www.sirc-csars.gc.ca/prddpr/is/2013/index-eng.html); Security and Intelligence Information Files – Personal Information Bank– PCO PPU 005 (http://www.pco-bcp.gc.ca/index.asp?lang=eng&amp;page=information&amp;sub=publications&amp;doc=info-source/index-eng.htm); Employee Personnel Record – PSE 901 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Governor in Council Appointments – PSU 918 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Members of Boards Committees and Councils – PSU 919 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Staffing – PSE 902 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp); Physical Access Controls PSU 907 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu907); Security – PRN 931 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-classes-records.html); Security Incidents and Privacy Breaches – PSU 939 (https://www.tbs-sct.gc.ca/hgw-cgf/oversight-surveillance/atip-aiprp/ai/spib-frpo-eng.asp)</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Au besoin, les renseignements personnels peuvent être communiqués conformément à la loi habilitante de l'institution et dans les paramètres de la Loi sur la protection des renseignements personnels, à la Gendarmerie royale du Canada ( Services canadiens d'identification criminelle en temps réel – GRC OPS 1214 et Fichiers sur la sécurité du personnel GRC ADM 445 ) et au Service canadien du renseignement de sécurité ( Évaluations de sécurité/Avis – SCRS PPU 005 ) pour qu’ils effectuent des vérifications, des enquêtes et/ou des évaluations de filtrage de sécurité, conformément à la Politique sur la sécurité du gouvernement. Les informations peuvent être communiquées à la Commission canadienne des droits de la personne ( Contentieux en matière de droits de la personne – CCDP REG 020 , Règlement des différends faisant l’objet d’une plainte — Droits de la personne – CCDP REG 010 ), Médiation des plaintes et des griefs – fichier de renseignements personnels – CRTFP OGP 579 ) , à la Commission des relations de travail et de l’emploi dans la fonction publique, au ministère de la Justice Canada ( Services de contentieux – JUS 3.0.5 ) ou au Comité de surveillance des activités de renseignement de sécurité ( Plaintes – SCA COM 001 ) lorsqu’une personne conteste une décision visant à refuser, à suspendre ou à révoquer une autorisation de sécurité ou une autorisation d’accès aux sites ou au Bureau du Conseil privé ( Fichiers d’information sur la sécurité et le renseignement – Fichier de renseignements personnels – BCP PPU 005 ) si la personne pose un risque potentiel à la sécurité nationale ou fait l’objet d’une enquête liée à la sécurité nationale. La cote de filtrage de sécurité d’une personne peut être communiquée à l’interne au sein des institutions aux responsables des ressources humaines afin de mettre à jour le dossier personnel de la personne concernée ( Dossier personnel d’un employé – POE 901, Nominations par le Gouverneur en conseil – POU 918 , Membres de conseils d’administration, de comités et de conseils – POU 919 ). Les informations peuvent être communiquées au sein d’une institution fédérale et entre elles aux fins de dotation ( Dotation – POE 902 ). Les informations peuvent être communiquées au sein des institutions aux responsables de la sécurité ministérielle pour la délivrance de cartes d’accès et de laissez-passer ( Contrôles d’accès physique – POU 907 ). Les informations peuvent être communiquées pour enquête au sein des institutions aux responsables de la sécurité ministérielle dans les cas d’informations préjudiciables ( Sécurité – NDP 931 ou Incidents de sécurité et atteintes à la vie privée – POU 939 ). Les informations peuvent être communiquées à des entités de l’extérieur de l’institution fédérale, y compris les bureaux de crédit pour qu’elles réalisent des enquêtes sur la situation financière. Les renseignements, y compris les résultats du filtrage de sécurité, peuvent être communiqués au gestionnaire d’une personne, aux conseillers en relations de travail, et/ou au conseil consultatif du filtrage de sécurité institutionnel, en fonction du besoin de savoir, lorsqu’une décision de refuser, de révoquer ou de suspendre en attente d’une enquête fait l’objet d’un examen. Les renseignements, y compris les formulaires d’enquête de sécurité dûment remplis, les résultats des vérifications du filtrage de sécurité et les décisions prises par un ministère peuvent être communiqués entre les responsables de sécurité institutionnels afin de permettre la transférabilité du filtrage de sécurité et d’aider à veiller à ce que les personnes ne soient pas engagées par une institution fédérale ou un ministère compte non tenu des circonstances menant à une révocation ou à un refus antérieur qui pourrait avoir eu lieu dans une autre institution. Certaines informations rendues anonymes peuvent être utilisées ou divulguées pour l’évaluation d’un programme.  |  Links: Services canadiens d'identification criminelle en temps réel – GRC OPS 1214 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-fra.htm); Fichiers sur la sécurité du personnel GRC ADM 445 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-fra.htm); Évaluations de sécurité/Avis – SCRS PPU 005 (https://www.csis.gc.ca/tp/nfsrc-fr.php); Contentieux en matière de droits de la personne – CCDP REG 020 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-fra.pdf); Règlement des différends faisant l’objet d’une plainte — Droits de la personne – CCDP REG 010 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-fra.pdf); Médiation des plaintes et des griefs – fichier de renseignements personnels – CRTFP OGP 579 (http://pslrb-crtfp.gc.ca/reports/1314/infosource_f.asp); Services de contentieux – JUS 3.0.5 (http://www.justice.gc.ca/fra/trans/aiprp-atip/infosource/p3.html); Plaintes – SCA COM 001 (http://www.sirc-csars.gc.ca/prddpr/is/2013/index-fra.html); Fichiers d’information sur la sécurité et le renseignement – Fichier de renseignements personnels – BCP PPU 005 (http://www.pco-bcp.gc.ca/index.asp?lang=fra&amp;page=information&amp;sub=publications&amp;doc=info-source/index-fra.htm); Dossier personnel d’un employé – POE 901, Nominations par le Gouverneur en conseil – POU 918 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/renseignements-programmes-fonds-renseignements/fichiers-renseignements-personnels-ordinaires.html); Membres de conseils d’administration, de comités et de conseils – POU 919 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/renseignements-programmes-fonds-renseignements/fichiers-renseignements-personnels-ordinaires.html); Dotation – POE 902 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/renseignements-programmes-fonds-renseignements/fichiers-renseignements-personnels-ordinaires.html); Contrôles d’accès physique – POU 907 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe907); Sécurité – NDP 931 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/renseignements-programmes-fonds-renseignements/categories-documents-ordinaires.html); Incidents de sécurité et atteintes à la vie privée – POU 939 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/renseignements-programmes-fonds-renseignements/fichiers-renseignements-personnels-ordinaires.html)</t>
+          <t>Au besoin, les renseignements personnels peuvent être communiqués conformément à la loi habilitante de l'institution et dans les paramètres de la Loi sur la protection des renseignements personnels, à la Gendarmerie royale du Canada ( Services canadiens d'identification criminelle en temps réel – GRC OPS 1214 et Fichiers sur la sécurité du personnel GRC ADM 445 ) et au Service canadien du renseignement de sécurité ( Évaluations de sécurité/Avis – SCRS PPU 005 ) pour qu’ils effectuent des vérifications, des enquêtes et/ou des évaluations de filtrage de sécurité, conformément à la Politique sur la sécurité du gouvernement. Les informations peuvent être communiquées à la Commission canadienne des droits de la personne ( Contentieux en matière de droits de la personne – CCDP REG 020 , Règlement des différends faisant l’objet d’une plainte — Droits de la personne – CCDP REG 010 ), Médiation des plaintes et des griefs – fichier de renseignements personnels – CRTFP OGP 579 ), à la Commission des relations de travail et de l’emploi dans la fonction publique, au ministère de la Justice Canada ( Services de contentieux – JUS 3.0.5 ) ou au Comité de surveillance des activités de renseignement de sécurité ( Plaintes – SCA COM 001 ) lorsqu’une personne conteste une décision visant à refuser, à suspendre ou à révoquer une autorisation de sécurité ou une autorisation d’accès aux sites ou au Bureau du Conseil privé ( Fichiers d’information sur la sécurité et le renseignement – Fichier de renseignements personnels – BCP PPU 005 ) si la personne pose un risque potentiel à la sécurité nationale ou fait l’objet d’une enquête liée à la sécurité nationale. La cote de filtrage de sécurité d’une personne peut être communiquée à l’interne au sein des institutions aux responsables des ressources humaines afin de mettre à jour le dossier personnel de la personne concernée ( Dossier personnel d’un employé – POE 901 , Nominations par le Gouverneur en conseil – POU 918 , Membres de conseils d’administration, de comités et de conseils – POU 919 ). Les informations peuvent être communiquées au sein d’une institution fédérale et entre elles aux fins de dotation ( Dotation – POE 902 ). Les informations peuvent être communiquées au sein des institutions aux responsables de la sécurité ministérielle pour la délivrance de cartes d’accès et de laissez-passer ( Contrôles d’accès physique – POU 907 ). Les informations peuvent être communiquées pour enquête au sein des institutions aux responsables de la sécurité ministérielle dans les cas d’informations préjudiciables ( Sécurité – NDP 931 ou Incidents de sécurité et atteintes à la vie privée – POU 939 ). Les informations peuvent être communiquées à des entités de l’extérieur de l’institution fédérale, y compris les bureaux de crédit pour qu’elles réalisent des enquêtes sur la situation financière. Les renseignements, y compris les résultats du filtrage de sécurité, peuvent être communiqués au gestionnaire d’une personne, aux conseillers en relations de travail, et/ou au conseil consultatif du filtrage de sécurité institutionnel, en fonction du besoin de savoir, lorsqu’une décision de refuser, de révoquer ou de suspendre en attente d’une enquête fait l’objet d’un examen. Les renseignements, y compris les formulaires d’enquête de sécurité dûment remplis, les résultats des vérifications du filtrage de sécurité et les décisions prises par un ministère peuvent être communiqués entre les responsables de sécurité institutionnels afin de permettre la transférabilité du filtrage de sécurité et d’aider à veiller à ce que les personnes ne soient pas engagées par une institution fédérale ou un ministère compte non tenu des circonstances menant à une révocation ou à un refus antérieur qui pourrait avoir eu lieu dans une autre institution. Certaines informations rendues anonymes peuvent être utilisées ou divulguées pour l’évaluation d’un programme.  |  Links: Services canadiens d'identification criminelle en temps réel – GRC OPS 1214 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-fra.htm); Fichiers sur la sécurité du personnel GRC ADM 445 (http://www.rcmp-grc.gc.ca/atip-aiprp/infosource/cor-cds-fra.htm); Évaluations de sécurité/Avis – SCRS PPU 005 (https://www.csis.gc.ca/tp/nfsrc-fr.php); Contentieux en matière de droits de la personne – CCDP REG 020 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-fra.pdf); Règlement des différends faisant l’objet d’une plainte — Droits de la personne – CCDP REG 010 (http://www.chrc-ccdp.gc.ca/sites/default/files/info_source2016-fra.pdf); Médiation des plaintes et des griefs – fichier de renseignements personnels – CRTFP OGP 579 (http://pslrb-crtfp.gc.ca/reports/1314/infosource_f.asp); Services de contentieux – JUS 3.0.5 (http://www.justice.gc.ca/fra/trans/aiprp-atip/infosource/p3.html); Plaintes – SCA COM 001 (http://www.sirc-csars.gc.ca/prddpr/is/2013/index-fra.html); Fichiers d’information sur la sécurité et le renseignement – Fichier de renseignements personnels – BCP PPU 005 (http://www.pco-bcp.gc.ca/index.asp?lang=fra&amp;page=information&amp;sub=publications&amp;doc=info-source/index-fra.htm); Dossier personnel d’un employé – POE 901 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe901); Nominations par le Gouverneur en conseil – POU 918 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou918); Membres de conseils d’administration, de comités et de conseils – POU 919 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou919); Dotation – POE 902 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe902); Contrôles d’accès physique – POU 907 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou907); Sécurité – NDP 931 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-renseignements-personnels/acces-information/info-source/categories-documents-ordinaires.html#ndp931); Incidents de sécurité et atteintes à la vie privée – POU 939 (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou939)</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -4609,6 +4783,9 @@
           <t>98/001</t>
         </is>
       </c>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr">
         <is>
           <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu917</t>
@@ -4636,6 +4813,7 @@
           <t>PSU 907</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>psu907</t>
@@ -4643,7 +4821,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>poe907</t>
+          <t>pou907</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -4676,6 +4854,7 @@
           <t>Ce fichier de renseignements personnels correspondait auparavant à deux fichiers de renseignements personnels distincts : Surveillance vidéo, registres de contrôle d’accès des visiteurs et laissez-passer POU 907 et Cartes d'identification et laissez-passer POE 917).</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
           <t>Employees, and those on assignment or contract and visitors who require access to a government institution or any other person within proximity of video surveillance recording capabilities.</t>
@@ -4701,6 +4880,7 @@
           <t>The  information may be used or disclosed to assist security officials in the  monitoring of activities and/or the issuance of access passes. Information may  be used for identification purposes in support of personnel security screening.  Information may be used to support compliance with other relevant Treasury Board policy instruments and policy directions. Additionally, records and recordings may record entry  and exit times from facilities and may be used in the event of security-related  incidents such as thefts or emergency situations. In such cases, this  information may be shared with appropriate law enforcement agencies, emergency  workers, appropriate staff relations officers, or investigative bodies for  further investigations, charges or disciplinary actions (refer to Security  Incidents and Privacy Breaches PSU 939 and Discipline  PSE 911 ). Video information that reveals evidence of illegal activity,  employee misconduct or accidents may be disclosed to appropriate staff  relations, facility owners, enforcement or investigative bodies for further  investigations, charges or disciplinary actions.  |  Links: Security  Incidents and Privacy Breaches PSU 939 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#psu939); Discipline  PSE 911 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/information-about-programs-information-holdings/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4738,7 +4918,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe907</t>
+          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#pou907</t>
         </is>
       </c>
     </row>
@@ -4758,6 +4938,7 @@
           <t>PSU 912</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>psu912</t>
@@ -4788,11 +4969,15 @@
           <t>Ce fichier décrit les renseignements contenus dans les ententes conclues entre les institutions fédérales, et une personne ou une société, afin de fournir des biens ou des services, de construire des ouvrages ou de louer des biens réels. Les renseignements personnels peuvent comprendre le nom, les coordonnées (y compris le nom commercial), les renseignements biographiques, les renseignements sur les études, les renseignements financiers, les évaluations/analyses, le numéro d’assurance sociale (NAS), un autre numéro d’identification (p. ex., numéro d’entreprise), et la signature.</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>Individuals representing themselves or employed through private companies (including temporary help services) who have submitted responses to Requests for Proposals and who have been engaged through contracts or standing offers with government institutions and individuals who are provided as professional references.</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
           <t>Personal information is used to manage the contracting process, which includes the request for and receipt of proposals, evaluation of bids, selection of contractor, preparation, negotiation, execution, and award of contract, the disbursement of funds for services, deliverables, or both as specified within the contract, and post-contract evaluation. For most government institutions, personal information is collected under the authority of the Financial Administration Act. For those institutions not subject to the Act, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority. The SIN is collected pursuant to the Income Tax Act.</t>
@@ -4808,6 +4993,7 @@
           <t>Information is used to maintain an inventory of potential contractors. Information may also be used to recover overpayments and debts owed to the Crown and, where applicable, to enable execution of orders of garnishment, attachment, or diversion of funds in accordance with the Garnishment, Attachment and Pension Diversion Act and related regulations. Information may be used to confirm the identity of contractors (where required) for access to governmental and institutional websites and databases and for the loan of equipment and/or supplies. Information, including the Social Insurance Number and Business Number, is disclosed to the Canada Revenue Agency in T4A-NR Supplementary and T1204 slips (refer to Individual Returns and Payment Processing – CRA PPU 005 and Business Returns and Payment Processing – CRA PPU 047 ) and the Province of Quebec (if applicable) for tax purposes. The information may be shared with/described in Standard Personal Information Banks Accounts Payable - PSU 931 and Accounts Receivable - PSU 932 for payment administration. Selected information on contracts for $10,000 or more, including the fact that a contractor is a former public servant in receipt of a Public Service Superannuation Act pension, may be made available on institutions’ websites, in compliance with proactive disclosure procedures. Information may also be used or disclosed for evaluation or reporting purposes.  |  Links: Individual Returns and Payment Processing – CRA PPU 005 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html); Business Returns and Payment Processing – CRA PPU 047 (http://www.cra-arc.gc.ca/gncy/tp/nfsrc/nfsrc-eng.html); Accounts Payable - PSU 931 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu931); Accounts Receivable - PSU 932 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu932)</t>
         </is>
       </c>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4865,6 +5051,7 @@
           <t>PSU 914</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>psu914</t>
@@ -4915,6 +5102,7 @@
           <t>Members of the public, representatives of private sector organizations and other government institutions (i.e., municipal, provincial/territorial, and international), employees and other representatives of government institutions, who have requested information from, or submitted information to, a government institution; parents and guardians of minors; employees and other individuals with access to institutional networks, including individuals who have prepared information for dissemination, such as publication on the institution’s extranet or internet sites or who act as contact points within the institution.</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
           <t>Personal information is used to disseminate information about the functions, programs, and activities of the institution, including about employees of the institution. For many institutions, personal information is collected under the authority of the Financial Administration Act (FAA), and in accordance with the Communications Policy of the Government of Canada. For those institutions not subject to the FAA or the Communications Policy of the Government of Canada, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority.</t>
@@ -4930,6 +5118,7 @@
           <t>The names, photographs, recordings and other personal information about individuals who work for the institution may be included in documentation posted on the institution’s extranet or Internet sites; e.g., within speeches, newsletters, etc. With consent of the individual, information may be shared with other areas of the institution for program-specific mailing/distribution lists and/or telephone lists. Information may be used to moderate public discussion on the social media platforms used by the institution. Responses to enquiries and any other relevant information are accounted for by the institution-specific personal information bank related to the program area that sent the response. Requests for information may be transferred when the requested information, e.g., inquiry or complaint, falls under the responsibility of another institution, refer to Executive Correspondence - PSU 902 . Some information may also be posted on government institutions’ websites for proactive disclosure purposes. Information may also be used or disclosed to provide statistical reports to management as well as for program evaluation.  |  Links: Executive Correspondence - PSU 902 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu902)</t>
         </is>
       </c>
+      <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -4987,6 +5176,7 @@
           <t>PSU 948</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>psu914a</t>
@@ -5017,6 +5207,9 @@
           <t>Ce fichier contient les renseignements liés à la gestion des biens immobiliers fédéraux et autres biens immobiliers utilisés ou acquis par une institution fédérale. Les biens immobiliers font référence à tout droit, intérêt ou profit dans des terres, y compris les mines, les minéraux et les améliorations qui leur sont apportées, sur ou sous terre. Les renseignements personnels peuvent comprendre le nom, les renseignements biographiques, les coordonnées, la taille de la famille, les antécédents en matière de crédit, les modalités relativement à la location, les renseignements financiers, les renseignements concernant les transactions liées à la propriété, y compris les évaluations, et une description de la propriété, y compris des photos.</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>Former or current tenants or applicants for tenancy of federal real property, real property owners, licensees, lessees, and property appraisers.</t>
@@ -5042,6 +5235,7 @@
           <t>Information may be used or disclosed for the following purposes: to collect debts owed by tenants as a result of their tenancy; for credit checks; for property tax payments, that is, information may be disclosed to municipalities in which the properties are located for tax assessments and administration of the payments-in-lieu of taxes program and for evaluation or reporting to senior management. Information may be shared with or described in the Standard Personal Information Banks Accounts Payable – PSU 931 , and Accounts Receivable – PSU 932 .  |  Links: Accounts Payable – PSU 931 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu931); Accounts Receivable – PSU 932 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu932)</t>
         </is>
       </c>
+      <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5099,6 +5293,7 @@
           <t>PSE 920</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>pse920</t>
@@ -5169,6 +5364,7 @@
           <t>The information may be used or disclosed for the following purposes: reporting to senior management, evaluation and audit. Some elements of the information may be published on the Internet, intranet or other medium. Information may be shared with PSE 904 Pay and Benefit in cases where awards qualify as income. Information may be shared with PSE 901 Employee Personnel Record.</t>
         </is>
       </c>
+      <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5226,6 +5422,7 @@
           <t>PSU 910</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>psu910</t>
@@ -5256,6 +5453,9 @@
           <t>Ces renseignements sont utilisés pour consigner des données sur les processus liés à la réinstallation d’employés et de leur famille. Les renseignements personnels recueillis comprennent le nom de la personne, le titre de son poste, le nom de son organisation, son numéro de téléphone au bureau et l’adresse du bureau, la classification et le niveau de son poste, son code d’identification de dossier personnel, le nom du fonctionnaire ou du gestionnaire de l’institution à qui les pouvoirs ont été délégués, des signatures, le nom de son conjoint ou de son conjoint de fait, le nom de ses enfants et de membres de sa famille élargie, ses besoins spéciaux sur le plan médical dont on pourrait avoir à tenir compte, ses relevés mensuels de cartes de crédit, ses déclarations personnelles de dépenses lorsqu’il n’est pas possible d’obtenir des reçus ou que les reçus ont été détruits par inadvertance, les coûts liés à son hypothèque ou à son loyer, les frais juridiques et les frais immobiliers.</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>Employees who relocate and their spouses or common-law partners, their children and/or extended family members. Also includes individuals representing third party suppliers, such as moving and storage companies.</t>
@@ -5281,6 +5481,7 @@
           <t>Non-personal information may be used to provide reports on employee relocations to management. The information may also be used for research, planning, audit and evaluation purposes.</t>
         </is>
       </c>
+      <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5296,6 +5497,7 @@
           <t>98/001 and 99/004</t>
         </is>
       </c>
+      <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr">
         <is>
           <t>PRN 936</t>
@@ -5470,6 +5672,7 @@
           <t>PSE 902</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>pse902</t>
@@ -5477,7 +5680,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>poe9021</t>
+          <t>poe902</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -5510,11 +5713,13 @@
           <t>Les personnes qui demandent des renseignements décrits dans ce fichier doivent fournir un numéro de concours, s’il y a lieu.</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>Employees of the institution and other individuals who apply for employment in the institution including through recruitment initiatives, as well as individuals who provide references or are supervisors of applicants.</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>Personal information is used to administer recruitment and staffing activities in government institutions, which includes maintaining an inventory of potential candidates for future staffing actions. For most government institutions, personal information is collected pursuant to the Public Service Employment Act, the Employment Equity Act, and the Canadian Human Rights Act (section 16). For those institutions not subject to these Acts, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority.</t>
@@ -5530,6 +5735,7 @@
           <t>Information may be disclosed to the Public Service Commission, Treasury Board Secretariat and other government institutions for recruitment, employment equity, and staffing purposes, including complaints (refer to Institution-Specific Personal Information Banks: for the Public Service Commission of Canada: Applicant Inventories and Referrals - PSC PPU 015 ; Assessment by the Personnel Psychology Centre - PSC PCU 025 , Second Language Evaluation (SLE) Test Results - PSC PPU 030 , Executive Resourcing - PSC PCE 746 , Analytical Environment - PSC PCE 761 , and Investigations, Mediation and Conciliation - PSC PPU 010 ; for Treasury Board of Canada Secretariat: Employment Equity Data Bank - TBS PCE 739 and Workforce Adjustment Monitoring (WFAM) System - TBS PCE 804 ). Information relating to staffing complaints may be shared with the Public Service Commission (refer to Institution-Specific Personal Information Bank Investigations, Mediation and Conciliation - PSC PPU 010 ) and the Federal Public Service Staffing Tribunal with Public Sector Labour Relations and Employment Board, when required. On request, selected information may be disclosed to a participant in a staffing process. Information may also be shared with third party service providers to manage recruitment initiatives. Information may also be used or disclosed for human resources planning and studies (refer to Standard Personal Information Bank Human Resources Planning - PSU 935 ) and staffing decisions may also be described in Standard Personal Information Bank Employee Personnel Record - PSE 901 . Voluntary self identification information relating to employment equity programs and services is also described in Standard Personal Information Bank Employment Equity and Diversity - PSE 918 . Selected information about reclassifications may be proactively disclosed on government institutions’ websites. Information may also be used or disclosed for program evaluation and reporting purposes.  |  Links: Applicant Inventories and Referrals - PSC PPU 015 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Assessment by the Personnel Psychology Centre - PSC PCU 025 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Second Language Evaluation (SLE) Test Results - PSC PPU 030 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Executive Resourcing - PSC PCE 746 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Analytical Environment - PSC PCE 761 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Investigations, Mediation and Conciliation - PSC PPU 010 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Employment Equity Data Bank - TBS PCE 739 (http://www.tbs-sct.gc.ca/atipo-baiprp/sfg-srg/sfg-srg02-eng.asp); Workforce Adjustment Monitoring (WFAM) System - TBS PCE 804 (http://www.tbs-sct.gc.ca/atipo-baiprp/sfg-srg/sfg-srg00-eng.asp); Investigations, Mediation and Conciliation - PSC PPU 010 (http://www.psc-cfp.gc.ca/abt-aps/atip-aiprp/infosource/2012/index-eng.htm); Human Resources Planning - PSU 935 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu935); Employee Personnel Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901); Employment Equity and Diversity - PSE 918 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse918)</t>
         </is>
       </c>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5567,7 +5773,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe9021</t>
+          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe902</t>
         </is>
       </c>
     </row>
@@ -5587,6 +5793,7 @@
           <t>PSE 905</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>pse905</t>
@@ -5617,11 +5824,15 @@
           <t>Ce fichier décrit les renseignements personnels recueillis à l’appui du programme de formation et de perfectionnement d’une institution (p. ex., les programmes de mentorat et d’orientation des carrières, les affectations et les modalités de travail de perfectionnement, etc.). Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements sur les études, le numéro d’identification d’employé, des renseignements sur l’équité en emploi, les renseignements personnels de l’employé, les renseignements financiers, les renseignements biographiques, ainsi que les résultats de l’analyse et de la formation.</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>Individuals who are employed by government institutions who register for training or development courses or programs.</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
           <t>Personal information is used to register and pay for approved training and development activities. Where applicable, government institutions may receive information from the Canada School of Public Service or other course providers about registration costs and training results. For most government institutions, personal information is collected under the authority of the Public Service Staff Relations Act and the Public Service Employment Act. For those institutions not subject to these Acts, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority.</t>
@@ -5637,6 +5848,7 @@
           <t>Information may be used to link voluntary self-identification data to information contained in other banks (refer to Standard Personal Information Bank Employment Equity and Diversity - PSE 918) for the purpose of implementing and evaluating government policies relating to employment equity and diversity. Some information may also be shared with/described in the Standard Personal Information Banks Accounts Receivable - PSU 932 , Employee Performance Management Program – PSE 912 and Employee Personnel Record - PSE 901 . Information may also be used or disclosed for program evaluation.  |  Links: Accounts Receivable - PSU 932 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu932); Employee Performance Management Program – PSE 912 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse912); Employee Personnel Record - PSE 901 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse901)</t>
         </is>
       </c>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5694,6 +5906,7 @@
           <t>PSU 909</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>psu909</t>
@@ -5724,11 +5937,15 @@
           <t>Ce fichier décrit les renseignements sur les employés qui se déplacent pour des activités officielles de leur institution. Les renseignements personnels peuvent comprendre le nom, les coordonnées, les renseignements biographiques, le numéro d’identification d’employé, les renseignements personnels de l’employé, les renseignements financiers et sur le passeport/visa, les antécédents de voyage, les demandes d’indemnité de voyages, le logement, les repas et les préférences. Les employés en voyages peuvent également être tenus de fournir la date de naissance et le sexe lorsqu’ils font des préparatifs de voyages.</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>Employees of government institutions, Ministers, Parliamentary Secretary, exempt staff, and other individuals (may include term or casual employees, temporary staff, volunteers, students, consultants and contractors, or witnesses) who travel on official institutional business, their spouses or common-law partners and dependants.</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
           <t>Personal information is used to process travel requirements for individuals who travel on behalf of the institution. For most government institutions, personal information is collected under the authority of the Financial Administration Act. For those institutions not subject to the Act, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority.</t>
@@ -5744,6 +5961,7 @@
           <t>Travel expenses incurred by the Minister, Parliamentary Secretary, exempt staff, and by senior level employees (i.e., Deputy Minister, Associate Deputy Minister, Assistant Deputy Minister, or equivalent) may be proactively disclosed on government institutions’ websites. Some institutions may share information with Public Works and Government Services Canada to establish the Traveller Profile (refer to Central Personal Information Bank Shared Travel Services Initiative (STSI) Traveller Profile - PWGSC PCE 706 ). In some instances, information may also be shared with the Department of Foreign Affairs and International Trade Canada (e.g., official delegations to events in foreign countries). Information may also be shared with/described in Standard Personal Information Banks Accounts Payable - PSU 931 and Accounts Receivable – PSU 93 2. Information may be used or disclosed for program evaluation and reporting purposes.  |  Links: Shared Travel Services Initiative (STSI) Traveller Profile - PWGSC PCE 706 (http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/index-eng.html); Accounts Payable - PSU 931 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu931); Accounts Receivable – PSU 93 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu932)</t>
         </is>
       </c>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5759,6 +5977,7 @@
           <t>98/001 and 99/004</t>
         </is>
       </c>
+      <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr">
         <is>
           <t>PRN 934, PRN 935</t>
@@ -5796,6 +6015,7 @@
           <t>PSE 915</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>pse915</t>
@@ -5846,6 +6066,7 @@
           <t>Current and former employees of government institutions, family members, and other individuals with whom the employee may have a business interest.</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
           <t>Personal information is used to provide direction and authorizations, support decision on transfers, discipline and termination of employment, if conflict of interest exists, resolve situations of perceived, potential and actual conflicts of interest in current and post-employment This includes conflicts of interest in relation to 1) assets and liabilities, 2) gifts, hospitality and other benefits, 3) outside employment or activities, 4) preferential treatment and 5) solicitation. Personal information is also used in assessing the need for the establishment of a blind trust or for approving reimbursement for costs associated with such a divestment. Personal information is collected pursuant to section 5 and 6 of the PSDPA. Personal information is collected pursuant to sections 7 and 11.1 (1)(j) of the Financial Administration Act (FAA) for setting terms and conditions of employment. For those institutions not subject to the PSDPA or the FAA, consult the institution’s Access to Information and Privacy Coordinator to determine collection authority.</t>
@@ -5861,6 +6082,7 @@
           <t>In some cases, information may be disclosed to the Office of the Chief Human Resources Officer, Treasury Board Secretariat for the purpose of obtaining advice on possible conflicts of interest. In cases where an allegation of wrongdoing is made, information may be disclosed either to the Office of the Public Sector Integrity Commissioner of Canada, which may make recommendations where warranted to Deputy Heads of institutions, refer to Case Review and Investigation Files – PSIO PPU 005 or to the senior officer responsible for receiving and dealing with disclosures of wrongdoing in the government institution, refer to Disclosure of Wrongdoing in the Workplace – PSU 906 . Information may be shared with human resources officials where a conflict of interest results in discipline or termination of employment, refer to Discipline – PSE 911 . Information may also be used or disclosed for program evaluation, policy analysis, research, audit or statistical purposes.  |  Links: Case Review and Investigation Files – PSIO PPU 005 (http://www.psic.gc.ca/eng/about-us/publications#ATIP); Disclosure of Wrongdoing in the Workplace – PSU 906 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#psu906); Discipline – PSE 911 (https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse911)</t>
         </is>
       </c>
+      <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5886,6 +6108,7 @@
           <t>PRN 920, PRN 926</t>
         </is>
       </c>
+      <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="inlineStr">
         <is>
           <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse915</t>
@@ -5913,6 +6136,7 @@
           <t>PSE 908</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>pse908</t>
@@ -5940,9 +6164,12 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Les dossiers contenant des renseignements décrits dans ce fichier peuvent comprendre des rapports sur les accidents; des réclamations pour les dommages subis; des décisions du tribunal; des règlements des transactions et la correspondance concernant des accidents survenus à des véhicules, des bateaux, des embarcations et des avions loués ou appartenant à l’état, ainsi qu’à des véhicules, bateaux, embarcations et avions privés utilisés à des fins professionnelles. Les dossiers de santé et sécurité au travail ainsi que les dossiers d’autorisation de congés et de prestations liés à une blessure au travail ou à une maladie professionnelle sont décrits dans le fichier de renseignements personnels ordinaire, Santé et sécurité au travail – POE 907.  |  Links: Santé et sécurité au travail – POE 907. (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe9071)</t>
-        </is>
-      </c>
+          <t>Les dossiers contenant des renseignements décrits dans ce fichier peuvent comprendre des rapports sur les accidents; des réclamations pour les dommages subis; des décisions du tribunal; des règlements des transactions et la correspondance concernant des accidents survenus à des véhicules, des bateaux, des embarcations et des avions loués ou appartenant à l’état, ainsi qu’à des véhicules, bateaux, embarcations et avions privés utilisés à des fins professionnelles. Les dossiers de santé et sécurité au travail ainsi que les dossiers d’autorisation de congés et de prestations liés à une blessure au travail ou à une maladie professionnelle sont décrits dans le fichier de renseignements personnels ordinaire, Santé et sécurité au travail – POE 907.  |  Links: Santé et sécurité au travail – POE 907. (https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe907)</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>Employees of the institution.</t>
@@ -5968,6 +6195,7 @@
           <t>To determine liability for such accidents and to approve damage settlements.</t>
         </is>
       </c>
+      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -5993,6 +6221,7 @@
           <t>PRN 922, PRN 945</t>
         </is>
       </c>
+      <c r="Y49" t="inlineStr"/>
       <c r="Z49" t="inlineStr">
         <is>
           <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#pse908</t>
@@ -6020,6 +6249,7 @@
           <t>PSE 930</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>pse930</t>
@@ -6050,6 +6280,9 @@
           <t>Les dossiers contenant les renseignements décrits dans ce fichier peuvent renfermer des renseignements recueillis à partir d’enquêtes menées par des institutions fédérales auprès de leurs employés pour évaluer la demande de garderies en milieu de travail, à partir des dossiers des garderies en milieu de travail. Ces renseignements ont été compilés dans le but de déterminer l’aide financière permanente sur laquelle pourront compter les garderies pour ce qui est de la location des locaux, et d’évaluer la politique sur les garderies. Ils peuvent comprendre des données personnelles sur l’employé ou l’utilisateur, ou encore sur ses enfants, et peuvent porter sur la demande prévue en services de garderie, la probabilité qu’un employé inscrive un enfant dans une garderie parrainée par l’institution et les raisons qui pourraient l’inciter à l’y inscrire.</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>All federal employees included in Schedules I and IV of the Financial Administration Act.</t>
@@ -6075,6 +6308,7 @@
           <t>The information in these records will be used for administrative and statistical purposes associated with the establishment of a day care centre. It will also be used for the evaluation and monitoring of the federal public service workplace day care policy. The information may be disclosed to Treasury Board, the government institution, an authorized committee of the government institution, a custodian government institution and the Board of Directors of the Day Care Centre. Together with the linked information from the files identified below, this information will form the basis for tabulations of the extent and type of employee day care users.</t>
         </is>
       </c>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
           <t>For information about the length of time that specific types of common administrative records are maintained by a government institution, including the final disposition of those records, please contact the institution’s Access to Information and Privacy Coordinator.</t>
@@ -6113,44 +6347,6 @@
       <c r="AA50" t="inlineStr">
         <is>
           <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#poe930</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>categories</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>categories</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>categories</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Categories of Personal Information</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Catégories de renseignements personnels</t>
-        </is>
-      </c>
-      <c r="Z51" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/standard-personal-information-banks.html#categories</t>
-        </is>
-      </c>
-      <c r="AA51" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/fichiers-renseignements-personnels-ordinaires.html#categories</t>
         </is>
       </c>
     </row>

</xml_diff>